<commit_message>
feat: crawl and populate all 20 products from hongcotsong.com with full metadata, images album, and multi-channel Google Sheet import mechanisms
</commit_message>
<xml_diff>
--- a/An-Cot-Song-du-lieu.xlsx
+++ b/An-Cot-Song-du-lieu.xlsx
@@ -33,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -45,8 +45,14 @@
       <b val="1"/>
       <color rgb="00FFFFFF"/>
     </font>
+    <font>
+      <name val="Segoe UI"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -56,6 +62,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="002B5675"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="002B5675"/>
+        <bgColor rgb="002B5675"/>
       </patternFill>
     </fill>
   </fills>
@@ -71,13 +83,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -543,7 +558,6 @@
           <t>model_spine_url</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -551,7 +565,6 @@
           <t>model_neck_url</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -559,7 +572,6 @@
           <t>model_joint_url</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -567,7 +579,6 @@
           <t>model_bp_url</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1796,125 +1807,2172 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N2"/>
+  <dimension ref="A1:T21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
-    <col width="30" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="30" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="30" customWidth="1" min="8" max="8"/>
-    <col width="30" customWidth="1" min="9" max="9"/>
-    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="10" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="40" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="18" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="18" customWidth="1" min="13" max="13"/>
+    <col width="16" customWidth="1" min="14" max="14"/>
+    <col width="16" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="16" max="16"/>
+    <col width="50" customWidth="1" min="17" max="17"/>
+    <col width="18" customWidth="1" min="18" max="18"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="3" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>price</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>currency</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>image_url</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t>video_url</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="3" t="inlineStr">
         <is>
           <t>buy_url</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>description</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="3" t="inlineStr">
         <is>
           <t>published</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="3" t="inlineStr">
         <is>
           <t>sort_order</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="3" t="inlineStr">
         <is>
           <t>button_label</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="3" t="inlineStr">
         <is>
           <t>button_class</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="3" t="inlineStr">
         <is>
           <t>video_button_label</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>video_button_class</t>
+        </is>
+      </c>
+      <c r="O1" s="3" t="inlineStr">
+        <is>
+          <t>display_layout</t>
+        </is>
+      </c>
+      <c r="P1" s="3" t="inlineStr">
+        <is>
+          <t>badge_label</t>
+        </is>
+      </c>
+      <c r="Q1" s="3" t="inlineStr">
+        <is>
+          <t>gallery_urls</t>
+        </is>
+      </c>
+      <c r="R1" s="3" t="inlineStr">
+        <is>
+          <t>chat_button_label</t>
+        </is>
+      </c>
+      <c r="S1" s="3" t="inlineStr">
+        <is>
+          <t>chat_button_url</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
+        <is>
+          <t>chat_button_class</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>goi-mau</t>
+          <t>goi-co-doctorloan-f5</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Gối hỗ trợ — sản phẩm minh họa</t>
+          <t>Gối cổ sáng chế DoctorLoan F5</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
-        <v>250000</v>
+        <v>4312000</v>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
           <t>VND</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr"/>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767624348098-149351903-goi-co-doctorloan-f5-1-scaled.jpg</t>
+        </is>
+      </c>
       <c r="F2" s="2" t="inlineStr"/>
-      <c r="G2" s="2" t="inlineStr"/>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/goi-co-sang-che-doctorloan-f5/</t>
+        </is>
+      </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>Dữ liệu minh họa. Quản trị viên thay bằng sản phẩm thực tế.</t>
+          <t>&lt;p&gt;Gối cổ sáng chế DOCTORLOAN F5 bảo vệ đường cong sinh lý và nắn chỉnh sai lệch đột sống cổ&lt;/p&gt;
+&lt;p&gt;ĐẶC ĐIỂM CỦA SẢN PHẨM&lt;/p&gt;
+&lt;p&gt;Đây là sản phẩm có công dụng hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cổ (thoát vị đĩa đệm, cong, vẹo, trật, trượt, thoái hóa, vôi hóa, gai xương), giúp điều chỉnh cột sống cổ trở lại trạng thái khỏe mạnh bình thường.&lt;/p&gt;
+&lt;p&gt;– Phần đầu thấp (9cm): Bảo vệ cấu trúc tự nhiên cột sống cổ ở cả tư thế nằm ngừa và nằm nghiêng. Với chất liệu mút có tỷ trọng rất cao nên có độ đàn hồi tốt, không bị xẹp lún, giữ đúng cấu trúc cổ trong suốt đêm khi ngủ. Phòng ngừa bệnh cột sống cổ, tạo giấc ngủ sâu, ngăn chặn bệnh mất ngủ. Dùng để ngủ, nghỉ ngơi và thư giãn&lt;/p&gt;
+&lt;p&gt;– Phần đầu cao (13cm): Có chứa một lõi cứng, không bị biến dạng dưới ảnh hưởng của trọng lực đè lên của cơ thể. Gối được thiết kế với độ dốc, chiều cao, chiều rộng bảo đảm việc sử dụng chính sức nặng của cơ thể để đẩy cột sống cổ về cấu trúc uốn cong và các đột sống trở lại vị trí bình thường. Kê 15- 30 phút mỗi lần. Mỗi ngày có thể kê nhiều lần&lt;/p&gt;
+&lt;p&gt;CÔNG DỤNG: Dùng đề giảm, mất dần và mất đi các triệu chứng như:&lt;/p&gt;
+&lt;p&gt;– Đau đầu, mệt mỏi, làm việc thiếu tập trung.&lt;/p&gt;
+&lt;p&gt;– Thiếu máu lên não, hoa mắt, chóng mặt, ù tai.&lt;/p&gt;
+&lt;p&gt;– Mờ mắt, méo mặt, méo mồm, suy giảm thính lực – Đau, tê, cứng, mỏi cổ vai gáy&lt;/p&gt;
+&lt;p&gt;– Đau vai, đau cánh tay; đau cổ tay, bàn tay, ngón tay.&lt;/p&gt;
+&lt;p&gt;Hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cổ:&lt;/p&gt;
+&lt;p&gt;– Thoát vị đĩa đệm&lt;/p&gt;
+&lt;p&gt;– Cong, vẹo, trật, trượt đốt sống&lt;/p&gt;
+&lt;p&gt;– Thoái hóa, vôi hóa, gai xương&lt;/p&gt;
+&lt;p&gt;– Giúp tạo hình lại đường cong sinh lý cổ, điều chỉnh cột sống cổ trở lại trạng thái khỏe mạnh bình thường&lt;/p&gt;
+&lt;p&gt;• CHẤT LIỆU:&lt;/p&gt;
+&lt;p&gt;– Ruột được làm từ PU foam.&lt;/p&gt;
+&lt;p&gt;– Lõi gối làm từ EPS foam hoặc PU đặc biệt&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc gối được làm từ vải kate thoáng mát mềm mịn&lt;/p&gt;
+&lt;p&gt;– Chịu lực lên đến 100 kg&lt;/p&gt;
+&lt;p&gt;KÍCH THƯỚC&lt;/p&gt;
+&lt;p&gt;– Dài x Rộng x Cao: 40 x 40 x 9/13 (cm)&lt;/p&gt;
+&lt;p&gt;– Khối lượng: 1 kg&lt;/p&gt;
+&lt;p&gt;BẢO HÀNH&lt;/p&gt;
+&lt;p&gt;-Ruột gối: 1 năm Lõi gối: 1 năm&lt;/p&gt;
+&lt;p&gt;-Vỏ gối: Không bảo hành.&lt;/p&gt;</t>
         </is>
       </c>
       <c r="I2" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J2" s="2" t="n">
         <v>1</v>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr"/>
+      <c r="M2" s="2" t="inlineStr"/>
+      <c r="N2" s="2" t="inlineStr"/>
+      <c r="O2" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P2" s="2" t="inlineStr">
+        <is>
+          <t>Gối sáng chế</t>
+        </is>
+      </c>
+      <c r="Q2" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768140456609-981819061-goi-co-doctorloan-f5-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140459224-381383911-goi-co-doctorloan-f5-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140464846-551561386-goi-co-doctorloan-f5-5-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140468875-866481899-goi-co-doctorloan-f5-6-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R2" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S2" s="2" t="inlineStr"/>
+      <c r="T2" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
+          <t>goi-co-doctorloan-f4</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Gối cổ sáng chế DoctorLoan F4</t>
+        </is>
+      </c>
+      <c r="C3" s="2" t="n">
+        <v>7624000</v>
+      </c>
+      <c r="D3" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767577003250-674779022-goi-co-doctorloan-f4-1-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F3" s="2" t="inlineStr"/>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/goi-co-sang-che-doctorloan-f4/</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Gối cổ sáng chế DOCTORLOAN F4 bảo vệ đường cong sinh lý và nắn chỉnh sai lệch đột sống cổ&lt;/p&gt;
+&lt;p&gt;ĐẶC ĐIỂM CỦA SẢN PHẨM&lt;/p&gt;
+&lt;p&gt;Đây là sản phẩm có công dụng hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cổ (thoát vị đĩa đệm, cong, vẹo, trật, trượt, thoái hóa, vôi hóa, gai xương), giúp điều chỉnh cột sống cổ trở lại trạng thái khỏe mạnh bình thường.&lt;/p&gt;
+&lt;p&gt;– Phần đầu thấp (9cm): Bảo vệ cấu trúc tự nhiên cột sống cổ ở cả tư thế nằm ngừa và nằm nghiêng. Với chất liệu mút có tỷ trọng rất cao nên có độ đàn hồi tốt, không bị xẹp lún, giữ đúng cấu trúc cổ trong suốt đêm khi ngủ. Phòng ngừa bệnh cột sống cổ, tạo giấc ngủ sâu, ngăn chặn bệnh mất ngủ. Dùng để ngủ, nghỉ ngơi và thư giãn&lt;/p&gt;
+&lt;p&gt;– Phần đầu cao (13cm): Có chứa một lõi cứng, không bị biến dạng dưới ảnh hưởng của trọng lực đè lên của cơ thể. Gối được thiết kế với độ dốc, chiều cao, chiều rộng bảo đảm việc sử dụng chính sức nặng của cơ thể để đẩy cột sống cổ về cấu trúc uốn cong và các đột sống trở lại vị trí bình thường. Kê 15- 30 phút mỗi lần. Mỗi ngày có thể kê nhiều lần&lt;/p&gt;
+&lt;p&gt;CÔNG DỤNG: Dùng đề giảm, mất dần và mất đi các triệu chứng như:&lt;/p&gt;
+&lt;p&gt;– Đau đầu, mệt mỏi, làm việc thiếu tập trung.&lt;/p&gt;
+&lt;p&gt;– Thiếu máu lên não, hoa mắt, chóng mặt, ù tai.&lt;/p&gt;
+&lt;p&gt;– Mờ mắt, méo mặt, méo mồm, suy giảm thính lực – Đau, tê, cứng, mỏi cổ vai gáy&lt;/p&gt;
+&lt;p&gt;– Đau vai, đau cánh tay; đau cổ tay, bàn tay, ngón tay.&lt;/p&gt;
+&lt;p&gt;Hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cổ:&lt;/p&gt;
+&lt;p&gt;– Thoát vị đĩa đệm&lt;/p&gt;
+&lt;p&gt;– Cong, vẹo, trật, trượt đốt sống&lt;/p&gt;
+&lt;p&gt;– Thoái hóa, vôi hóa, gai xương&lt;/p&gt;
+&lt;p&gt;– Giúp tạo hình lại đường cong sinh lý cổ, điều chỉnh cột sống cổ trở lại trạng thái khỏe mạnh bình thường&lt;/p&gt;
+&lt;p&gt;• CHẤT LIỆU:&lt;/p&gt;
+&lt;p&gt;– Ruột được làm từ PU foam.&lt;/p&gt;
+&lt;p&gt;– Lõi gối làm từ EPS foam hoặc PU đặc biệt&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc gối được làm từ vải kate thoáng mát mềm mịn&lt;/p&gt;
+&lt;p&gt;– Chịu lực lên đến 100 kg&lt;/p&gt;
+&lt;p&gt;KÍCH THƯỚC&lt;/p&gt;
+&lt;p&gt;– Dài x Rộng x Cao: 40 x 40 x 9/13 (cm)&lt;/p&gt;
+&lt;p&gt;– Khối lượng: 1 kg&lt;/p&gt;
+&lt;p&gt;BẢO HÀNH&lt;/p&gt;
+&lt;p&gt;-Ruột gối: 1 năm Lõi gối: 1 năm&lt;/p&gt;
+&lt;p&gt;-Vỏ gối: Không bảo hành.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="K3" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L3" s="2" t="inlineStr"/>
+      <c r="M3" s="2" t="inlineStr"/>
+      <c r="N3" s="2" t="inlineStr"/>
+      <c r="O3" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P3" s="2" t="inlineStr">
+        <is>
+          <t>Gối sáng chế</t>
+        </is>
+      </c>
+      <c r="Q3" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767577012969-211026264-goi-co-doctorloan-f4-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140497963-707220928-goi-co-doctorloan-f4-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140500895-370706163-goi-co-doctorloan-f4-4-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140503751-489860843-goi-co-doctorloan-f4-5-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140506945-505448298-goi-co-doctorloan-f4-6-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R3" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S3" s="2" t="inlineStr"/>
+      <c r="T3" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>goi-co-doctorloan-f6</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Gối cổ sáng chế DoctorLoan F6</t>
+        </is>
+      </c>
+      <c r="C4" s="2" t="n">
+        <v>7049000</v>
+      </c>
+      <c r="D4" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767624241501-394241632-goi-co-doctorloan-f6-0-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F4" s="2" t="inlineStr"/>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/goi-co-sang-che-doctorloan-f6/</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Gối cổ sáng chế DOCTORLOAN F6 bảo vệ đường cong sinh lý và nắn chỉnh sai lệch đột sống cổ&lt;/p&gt;
+&lt;p&gt;ĐẶC ĐIỂM CỦA SẢN PHẨM&lt;/p&gt;
+&lt;p&gt;Đây là sản phẩm có công dụng hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cổ (thoát vị đĩa đệm, cong, vẹo, trật, trượt, thoái hóa, vôi hóa, gai xương), giúp điều chỉnh cột sống cổ trở lại trạng thái khỏe mạnh bình thường.&lt;/p&gt;
+&lt;p&gt;– Phần đầu thấp (9cm): Bảo vệ cấu trúc tự nhiên cột sống cổ ở cả tư thế nằm ngừa và nằm nghiêng. Với chất liệu mút có tỷ trọng rất cao nên có độ đàn hồi tốt, không bị xẹp lún, giữ đúng cấu trúc cổ trong suốt đêm khi ngủ. Phòng ngừa bệnh cột sống cổ, tạo giấc ngủ sâu, ngăn chặn bệnh mất ngủ. Dùng để ngủ, nghỉ ngơi và thư giãn&lt;/p&gt;
+&lt;p&gt;– Phần đầu cao (13cm): Có chứa một lõi cứng, không bị biến dạng dưới ảnh hưởng của trọng lực đè lên của cơ thể. Gối được thiết kế với độ dốc, chiều cao, chiều rộng bảo đảm việc sử dụng chính sức nặng của cơ thể để đẩy cột sống cổ về cấu trúc uốn cong và các đột sống trở lại vị trí bình thường. Kê 15- 30 phút mỗi lần. Mỗi ngày có thể kê nhiều lần&lt;/p&gt;
+&lt;p&gt;CÔNG DỤNG: Dùng đề giảm, mất dần và mất đi các triệu chứng như:&lt;/p&gt;
+&lt;p&gt;– Đau đầu, mệt mỏi, làm việc thiếu tập trung.&lt;/p&gt;
+&lt;p&gt;– Thiếu máu lên não, hoa mắt, chóng mặt, ù tai.&lt;/p&gt;
+&lt;p&gt;– Mờ mắt, méo mặt, méo mồm, suy giảm thính lực – Đau, tê, cứng, mỏi cổ vai gáy&lt;/p&gt;
+&lt;p&gt;– Đau vai, đau cánh tay; đau cổ tay, bàn tay, ngón tay.&lt;/p&gt;
+&lt;p&gt;Hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cổ:&lt;/p&gt;
+&lt;p&gt;– Thoát vị đĩa đệm&lt;/p&gt;
+&lt;p&gt;– Cong, vẹo, trật, trượt đốt sống&lt;/p&gt;
+&lt;p&gt;– Thoái hóa, vôi hóa, gai xương&lt;/p&gt;
+&lt;p&gt;– Giúp tạo hình lại đường cong sinh lý cổ, điều chỉnh cột sống cổ trở lại trạng thái khỏe mạnh bình thường&lt;/p&gt;
+&lt;p&gt;• CHẤT LIỆU:&lt;/p&gt;
+&lt;p&gt;– Ruột được làm từ PU foam.&lt;/p&gt;
+&lt;p&gt;– Lõi gối làm từ EPS foam hoặc PU đặc biệt&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc gối được làm từ vải kate thoáng mát mềm mịn&lt;/p&gt;
+&lt;p&gt;– Chịu lực lên đến 100 kg&lt;/p&gt;
+&lt;p&gt;KÍCH THƯỚC&lt;/p&gt;
+&lt;p&gt;– Dài x Rộng x Cao: 40 x 40 x 9/13 (cm)&lt;/p&gt;
+&lt;p&gt;– Khối lượng: 1 kg&lt;/p&gt;
+&lt;p&gt;BẢO HÀNH&lt;/p&gt;
+&lt;p&gt;-Ruột gối: 1 năm Lõi gối: 1 năm&lt;/p&gt;
+&lt;p&gt;-Vỏ gối: Không bảo hành.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J4" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="K4" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L4" s="2" t="inlineStr"/>
+      <c r="M4" s="2" t="inlineStr"/>
+      <c r="N4" s="2" t="inlineStr"/>
+      <c r="O4" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P4" s="2" t="inlineStr">
+        <is>
+          <t>Gối sáng chế</t>
+        </is>
+      </c>
+      <c r="Q4" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768140476127-803637101-goi-co-doctorloan-f6-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140478988-600179260-goi-co-doctorloan-f6-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140482313-129339749-goi-co-doctorloan-f6-4-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140485758-827880909-goi-co-doctorloan-f6-5-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140488169-266575898-goi-co-doctorloan-f6-6-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R4" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S4" s="2" t="inlineStr"/>
+      <c r="T4" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>goi-lung-doctorloan-f1</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>Gối lưng sáng chế DoctorLoan F1 (Gối Dài)</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>1868000</v>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767624564646-522408653-goi-lung-doctorloan-f1-1-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr"/>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/goi-lung-sang-che-doctorloan-f1-goi-dai/</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Gối lưng sáng chế DoctorLoan F1 giúp bảo vệ và nắn chỉnh lại các sai lệch đốt sống lưng, ngực&lt;/p&gt;
+&lt;p&gt;ĐẶC ĐIỂM&lt;/p&gt;
+&lt;p&gt;– Đây là sản phẩm có công dụng hỗ trợ điều trị và ngăn ngừa các bệnh cột sống lưng (thoát vị đĩa đệm, cong, vẹo, trật, trượt, thoái hóa, vôi hóa, gai xương, mất đường cong sinh lý), giúp điều chỉnh cột sống lưng, cột sống ngực trở lại trạng thái khỏe mạnh bình thường.&lt;/p&gt;
+&lt;p&gt;– Phần lõi của gối có tính chịu sức ép cao, không biến đổi hình dạng dưới lực đè mạnh. Khi nằm lên gối sẽ sử dụng chính sức nặng cơ thể để nắn chỉnh, tạo hình lại đường cong sinh lý lưng và ngực, nắn chỉnh các đốt sống lưng, ngực trở về vị trí bình thường.&lt;/p&gt;
+&lt;p&gt;– Gối giúp giảm các triệu chứng đau, nhức, mỏi, tê vùng ngực – lưng. Cải thiện hiệu quả với những người bị thoái hoá đốt sống lưng, thoát vị đĩa đệm, cong vẹo cột sống, mất đường cong sinh lý đốt sống lưng.&lt;/p&gt;
+&lt;p&gt;CÔNG DỤNG: Giúp giảm nhanh các triệu chứng&lt;/p&gt;
+&lt;p&gt;– Đau cấp tính thắt lưng, mông, chân khi vận động sai tư thế&lt;/p&gt;
+&lt;p&gt;– Đau lưng dữ dội hoặc âm ỉ kéo dài do: đau thần kinh toạ, đau thoát vị đĩa đệm cột sống lưng, trật vẹo cột sống thắt lưng&lt;/p&gt;
+&lt;p&gt;– Đau/ nhói ngực, khó thở do biến đổi cấu trúc cột sống ngực&lt;/p&gt;
+&lt;p&gt;– Đau do xương chậu và xương cùng bị biến dạng do nằm sai tư thế trong sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p&gt;– Tê / buốt/ mất cảm giác chân, ngón chân&lt;/p&gt;
+&lt;p&gt;ĐỐI TƯỢNG SỬ DỤNG Gối lưng sáng chế DOCTORLOAN F1 dành cho mọi đối tượng từ trẻ em đến người già. Gối có chiều cao thấp nên nắn chỉnh chậm và an toàn. Phù hợp với cả những người đã từng phẫu thuật.&lt;/p&gt;
+&lt;p&gt;CÁCH SỬ DỤNG&lt;/p&gt;
+&lt;p&gt;– Kê lưng qua đêm khi ngủ.&lt;/p&gt;
+&lt;p&gt;– Kê lưng khi tập thể hình. Kê lưng khi đi tàu xe, máy bay.&lt;/p&gt;
+&lt;p&gt;CHẤT LIỆU&lt;/p&gt;
+&lt;p&gt;– Ruột được làm từ PU foam&lt;/p&gt;
+&lt;p&gt;– Lõi gối làm từ EPS foam hoặc PU đặc biệt&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc gối được làm từ vải kate thoáng mát mềm mịn&lt;/p&gt;
+&lt;p&gt;– Chịu lực lên đến 100 kg KÍCH THƯỚC&lt;/p&gt;
+&lt;p&gt;– Gối ngắn (Size S): 40 x 15 x 7 (cm). Khối lượng: 0,3 kg&lt;/p&gt;
+&lt;p&gt;– Gối dài dài (Size L): 50 x 15 x 7 (cm). Khối lượng: 0,3 kg&lt;/p&gt;
+&lt;p&gt;BẢO HÀNH&lt;/p&gt;
+&lt;p&gt;– Ruột gối và lõi gối: 1 năm&lt;/p&gt;
+&lt;p&gt;– Vỏ gối: Không bảo hành&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
+      <c r="N5" s="2" t="inlineStr"/>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P5" s="2" t="inlineStr">
+        <is>
+          <t>Gối sáng chế</t>
+        </is>
+      </c>
+      <c r="Q5" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768140380180-979017498-goi-lung-doctorloan-f1-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140382557-153705806-goi-lung-doctorloan-f1-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140389731-278672171-goi-lung-doctorloan-f1-4-1-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768833493819-989924893-goi-lung-doctorloan-f1-5-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R5" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S5" s="2" t="inlineStr"/>
+      <c r="T5" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>goi-lung-doctorloan-f3</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>Gối lưng sáng chế DoctorLoan F3</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3737000</v>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767624380299-768343988-goi-lung-doctorloan-f3-1-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr"/>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/goi-lung-sang-che-doctorloan-f3/</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Gối lưng sáng chế DoctorLoan F3 giúp bảo vệ và nắn chỉnh lại các sai lệch đốt sống lưng, ngực&lt;/p&gt;
+&lt;p&gt;ĐẶC ĐIỂM&lt;/p&gt;
+&lt;p&gt;– Đây là sản phẩm có công dụng hỗ trợ điều trị và ngăn ngừa các bệnh cột sống lưng (thoát vị đĩa đệm, cong, vẹo, trật, trượt, thoái hóa, vôi hóa, gai xương, mất đường cong sinh lý), giúp điều chỉnh cột sống lưng, cột sống ngực trở lại trạng thái khỏe mạnh bình thường.&lt;/p&gt;
+&lt;p&gt;– Phần lõi của gối có tính chịu sức ép cao, không biến đổi hình dạng dưới lực đè mạnh. Khi nằm lên gối sẽ sử dụng chính sức nặng cơ thể để nắn chỉnh, tạo hình lại đường cong sinh lý lưng và ngực, nắn chỉnh các đốt sống lưng, ngực trở về vị trí bình thường.&lt;/p&gt;
+&lt;p&gt;– Gối giúp giảm các triệu chứng đau, nhức, mỏi, tê vùng ngực – lưng. Cải thiện hiệu quả với những người bị thoái hoá đốt sống lưng, thoát vị đĩa đệm, cong vẹo cột sống, mất đường cong sinh lý đốt sống lưng.&lt;/p&gt;
+&lt;p&gt;CÔNG DỤNG: Giúp giảm nhanh các triệu chứng&lt;/p&gt;
+&lt;p&gt;– Đau cấp tính thắt lưng, mông, chân khi vận động sai tư thế&lt;/p&gt;
+&lt;p&gt;– Đau lưng dữ dội hoặc âm ỉ kéo dài do: đau thần kinh toạ, đau thoát vị đĩa đệm cột sống lưng, trật vẹo cột sống thắt lưng&lt;/p&gt;
+&lt;p&gt;– Đau/ nhói ngực, khó thở do biến đổi cấu trúc cột sống ngực&lt;/p&gt;
+&lt;p&gt;– Đau do xương chậu và xương cùng bị biến dạng do nằm sai tư thế trong sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p&gt;– Tê / buốt/ mất cảm giác chân, ngón chân&lt;/p&gt;
+&lt;p&gt;ĐỐI TƯỢNG SỬ DỤNG&lt;/p&gt;
+&lt;p&gt;Gối lưng sáng chế DOCTORLOAN F4 dành cho mọi đối tượng ngoại trừ người già bị loãng xương. Những trường hợp đặc biệt (đã từng mổ thay đĩa đệm, bắt vít cột sống) phải có chỉ định của bác sĩ.&lt;/p&gt;
+&lt;p&gt;CÁCH SỬ DỤNG Kê lưng 20 phút mỗi lần, một ngày 3-4 lần.&lt;/p&gt;
+&lt;p&gt;CHẤT LIỆU&lt;/p&gt;
+&lt;p&gt;– Ruột được làm từ PU foam&lt;/p&gt;
+&lt;p&gt;– Lõi gối làm từ EPS foam hoặc PU đặc biệt&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc gối được làm từ vải kate thoáng mát mềm mịn&lt;/p&gt;
+&lt;p&gt;– Chịu lực lên đến 100 kg&lt;/p&gt;
+&lt;p&gt;KÍCH THƯỚC&lt;/p&gt;
+&lt;p&gt;– Dài x rộng x cao: 48 x 25 x 10,5 (cm)&lt;/p&gt;
+&lt;p&gt;– Khối lượng: 0,5 kg&lt;/p&gt;
+&lt;p&gt;BẢO HÀNH&lt;/p&gt;
+&lt;p&gt;– Ruột gối và lõi gối: 1 năm&lt;/p&gt;
+&lt;p&gt;– Vỏ gối: Không bảo hành&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="K6" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr"/>
+      <c r="M6" s="2" t="inlineStr"/>
+      <c r="N6" s="2" t="inlineStr"/>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>Gối sáng chế</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768140445042-521234568-goi-lung-doctorloan-f3-5-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140438213-336026561-goi-lung-doctorloan-f3-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140440646-713627241-goi-lung-doctorloan-f3-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140443068-271317917-goi-lung-doctorloan-f3-4-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr"/>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>goi-lung-doctorloan-f4</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>Gối lưng sáng chế DoctorLoan F4</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3737000</v>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768140408734-365136374-goi-lung-doctorloan-f4-1-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr"/>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/goi-lung-sang-che-doctorloan-f4/</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Gối lưng sáng chế DoctorLoan F4 giúp bảo vệ và nắn chỉnh lại các sai lệch đốt sống lưng, ngực&lt;/p&gt;
+&lt;p&gt;ĐẶC ĐIỂM&lt;/p&gt;
+&lt;p&gt;– Đây là sản phẩm có công dụng hỗ trợ điều trị và ngăn ngừa các bệnh cột sống lưng (thoát vị đĩa đệm, cong, vẹo, trật, trượt, thoái hóa, vôi hóa, gai xương, mất đường cong sinh lý), giúp điều chỉnh cột sống lưng, cột sống ngực trở lại trạng thái khỏe mạnh bình thường.&lt;/p&gt;
+&lt;p&gt;– Phần lõi của gối có tính chịu sức ép cao, không biến đổi hình dạng dưới lực đè mạnh. Khi nằm lên gối sẽ sử dụng chính sức nặng cơ thể để nắn chỉnh, tạo hình lại đường cong sinh lý lưng và ngực, nắn chỉnh các đốt sống lưng, ngực trở về vị trí bình thường.&lt;/p&gt;
+&lt;p&gt;– Gối giúp giảm các triệu chứng đau, nhức, mỏi, tê vùng ngực – lưng. Cải thiện hiệu quả với những người bị thoái hoá đốt sống lưng, thoát vị đĩa đệm, cong vẹo cột sống, mất đường cong sinh lý đốt sống lưng.&lt;/p&gt;
+&lt;p&gt;CÔNG DỤNG: Giúp giảm nhanh các triệu chứng&lt;/p&gt;
+&lt;p&gt;– Đau cấp tính thắt lưng, mông, chân khi vận động sai tư thế&lt;/p&gt;
+&lt;p&gt;– Đau lưng dữ dội hoặc âm ỉ kéo dài do: đau thần kinh toạ, đau thoát vị đĩa đệm cột sống lưng, trật vẹo cột sống thắt lưng&lt;/p&gt;
+&lt;p&gt;– Đau/ nhói ngực, khó thở do biến đổi cấu trúc cột sống ngực&lt;/p&gt;
+&lt;p&gt;– Đau do xương chậu và xương cùng bị biến dạng do nằm sai tư thế trong sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p&gt;– Tê / buốt/ mất cảm giác chân, ngón chân&lt;/p&gt;
+&lt;p&gt;ĐỐI TƯỢNG SỬ DỤNG&lt;/p&gt;
+&lt;p&gt;Gối lưng sáng chế DOCTORLOAN F4 dành cho mọi đối tượng ngoại trừ người già bị loãng xương. Những trường hợp đặc biệt (đã từng mổ thay đĩa đệm, bắt vít cột sống) phải có chỉ định của bác sĩ.&lt;/p&gt;
+&lt;p&gt;CÁCH SỬ DỤNG Kê lưng 20 phút mỗi lần, một ngày 3-4 lần.&lt;/p&gt;
+&lt;p&gt;CHẤT LIỆU&lt;/p&gt;
+&lt;p&gt;– Ruột được làm từ PU foam&lt;/p&gt;
+&lt;p&gt;– Lõi gối làm từ EPS foam hoặc PU đặc biệt&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc gối được làm từ vải kate thoáng mát mềm mịn&lt;/p&gt;
+&lt;p&gt;– Chịu lực lên đến 100 kg&lt;/p&gt;
+&lt;p&gt;KÍCH THƯỚC&lt;/p&gt;
+&lt;p&gt;– Dài x rộng x cao: 48 x 25 x 10,5 (cm)&lt;/p&gt;
+&lt;p&gt;– Khối lượng: 0,5 kg&lt;/p&gt;
+&lt;p&gt;BẢO HÀNH&lt;/p&gt;
+&lt;p&gt;– Ruột gối và lõi gối: 1 năm&lt;/p&gt;
+&lt;p&gt;– Vỏ gối: Không bảo hành&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr"/>
+      <c r="M7" s="2" t="inlineStr"/>
+      <c r="N7" s="2" t="inlineStr"/>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>Gối sáng chế</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768140419864-514756467-goi-lung-doctorloan-f4-4-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140411610-502332487-goi-lung-doctorloan-f4-2-1-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140414551-726188349-goi-lung-doctorloan-f4-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140417023-50306941-goi-lung-doctorloan-f4-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140422559-802203686-goi-lung-doctorloan-f4-5-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr"/>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>ghe-doctorloan-n85-chan-ngan</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế DoctorLoan N85 (Chân Ngắn)</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>2127000</v>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767625485274-276617036-ghe-doctorloan-N85-1-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr"/>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/ghe-sang-che-doctorloan-n85-chan-ngan/</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Ghế sáng chế DoctorLoan N85 giữ dáng ngồi chuẩn, bảo vệ cấu trúc cột sống&lt;/p&gt;
+&lt;p&gt;ĐẶC ĐIỂM:&lt;/p&gt;
+&lt;p&gt;-Ghế Sáng chế DOCTORLOAN N85 là giải pháp điều chỉnh xương chậu luôn ở tư thế thẳng và cân xứng khi ngồi, từ đó bảo vệ cột sống trong hình dạng tốt nhất cho nhiều đối tượng khác nhau.&lt;/p&gt;
+&lt;p&gt;-Với những người đã bị biến dạng cột sống hoặc bệnh vẹo cột sống bẩm sinh thì ghế sáng chế DOCTORLOAN N85 ngăn chặn yêu tố gây tiến triển nặng của bệnh bởi cơ chế ÔM CHẶT&lt;/p&gt;
+&lt;p&gt;-GIỮ CHUẨN&lt;/p&gt;
+&lt;p&gt;– CHỐNG TRƯỢT. THIẾT KẾ VƯỢT TRỘI&lt;/p&gt;
+&lt;p&gt;-Thiết kế lưng ghế: Độ ngả của lưng ghế theo đường cong tự nhiên của cột sống, giúp người ngồi đúng tư thế thẳng mà vẫn có điểm tựa thoải mái. Trụ lưng ghế vững chắc nhờ những đường gân gia cường giúp ghế bền chắc với thời gian.&lt;/p&gt;
+&lt;p&gt;-Thiết kế mặt ghế: “Phần lồi phía trước mặt ghế” giữ cho xương chậu thẳng đứng, không bị trượt đổ nghiêng (hiện tượng ngồi trượt mông ra trước). Xương chậu được ví như móng nhà trong cơ thể, khi xương chậu bị đổ nghiêng sẽ gây ra biến dạng cột sống, tăng sức ép trên đĩa đệm gây thoát vị đĩa đệm.&lt;/p&gt;
+&lt;p&gt;-Thiết kế lồi ở phần lưng, lõm ở phần mông và phần lồi ở mặt ghế tạo ra khối cấu trúc LOCK – HOLD ÔM CHẶT – GIỮ CHUẨN – CHỐNG TRƯỢT.&lt;/p&gt;
+&lt;p&gt;-Kích thước mặt ghế là 35cm, ngắn hơn ghế thông thường: đây là một điểm khác biệt có ưu thế giúp áp chặt lưng vào khối ÔM CHẶT – GIỮ CHUẢN – CHỐNG TRƯỢT. Thích hợp với chiều cao khác nhau của nhiều người, giúp hai chân đặt vững trên mặt đất.&lt;/p&gt;
+&lt;p&gt;TÁC DỤNG SẢN PHẨM&lt;/p&gt;
+&lt;p&gt;-Dùng để ngồi làm việc, học tập, sinh hoạt hàng ngày. Đồng thời có tác dụng ĐIỀU CHỈNH XƯƠNG CHẬU, XƯƠNG CÙNG, XƯƠNG SỐNG VỀ HÌNH DẠNG BÌNH THƯỜNG.&lt;/p&gt;
+&lt;p&gt;-Hiệu quả khi sử dụng: Phòng ngừa LỆCH VẸO và các bệnh cột sống phát sinh do ngồi sai tư thế.&lt;/p&gt;
+&lt;p&gt;-Ghế ngồi sáng chế DOCTORLOAN N85 cần thiết cho mọi người, mọi lúc, mọi nơi, trong sinh hoạt hằng ngày nhằm phòng ngừa bệnh cột sống do ngồi sai tư thế.&lt;/p&gt;
+&lt;p&gt;-Sản phẩm phù hợp sử dụng ở mọi nơi như trong gia đình, bệnh viện, phòng khám, trường học, sân bay, văn phòng làm việc và ngoài trời (sân vận động, trạm xe buýt, ). CHẤT LIỆU: -Nhựa PP nguyên sinh 100%&lt;/p&gt;
+&lt;p&gt;-Khả năng chịu lực lên đến 150 kg&lt;/p&gt;
+&lt;p&gt;BẢO HÀNH:&lt;/p&gt;
+&lt;p&gt;-Chân ghế: 3 năm&lt;/p&gt;
+&lt;p&gt;-Thân ghế: 3 năm -Màu sắc: 1 năm theo tiêu chuẩn nhà sản xuất CÁCH CHỌN CHÂN GHẾ N85&lt;/p&gt;
+&lt;p&gt;– Ghế chân ngắn: dành cho người cao 1m45-1m75 ngồi với bàn 75cm. Nếu cao dưới 1m45 cần có bàn nâng hạ chiều cao&lt;/p&gt;
+&lt;p&gt;– Ghế chân dài: dành cho người cao trên 1m75 và cao dưới 1m45 ngồi với bàn cố định 75cm.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="K8" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr"/>
+      <c r="M8" s="2" t="inlineStr"/>
+      <c r="N8" s="2" t="inlineStr"/>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768140196380-790395769-ghe-doctorloan-N85-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140199100-761249413-ghe-doctorloan-N85-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140202131-796146365-ghe-doctorloan-N85-4-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140204796-669319825-ghe-doctorloan-N85-5-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140207980-580567712-ghe-doctorloan-N85-6-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr"/>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>ghe-doctorloan-n85-chan-dai</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế DoctorLoan N85 (Chân Dài)</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>2300000</v>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768818007231-277978911-ghe-doctorloan-N85-1-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr"/>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/dong-xuan-1ghe-sang-che-doctorloan-n85-chan-dai/</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Ghế sáng chế DoctorLoan N85 giữ dáng ngồi chuẩn, bảo vệ cấu trúc cột sống&lt;/p&gt;
+&lt;p&gt;ĐẶC ĐIỂM:&lt;/p&gt;
+&lt;p&gt;-Ghế Sáng chế DOCTORLOAN N85 là giải pháp điều chỉnh xương chậu luôn ở tư thế thẳng và cân xứng khi ngồi, từ đó bảo vệ cột sống trong hình dạng tốt nhất cho nhiều đối tượng khác nhau.&lt;/p&gt;
+&lt;p&gt;-Với những người đã bị biến dạng cột sống hoặc bệnh vẹo cột sống bẩm sinh thì ghế sáng chế DOCTORLOAN N85 ngăn chặn yêu tố gây tiến triển nặng của bệnh bởi cơ chế ÔM CHẶT -GIỮ CHUẨN – CHỐNG TRƯỢT.&lt;/p&gt;
+&lt;p&gt;THIẾT KẾ VƯỢT TRỘI&lt;/p&gt;
+&lt;p&gt;-Thiết kế lưng ghế: Độ ngả của lưng ghế theo đường cong tự nhiên của cột sống, giúp người ngồi đúng tư thế thẳng mà vẫn có điểm tựa thoải mái. Trụ lưng ghế vững chắc nhờ những đường gân gia cường giúp ghế bền chắc với thời gian.&lt;/p&gt;
+&lt;p&gt;-Thiết kế mặt ghế: “Phần lồi phía trước mặt ghế” giữ cho xương chậu thẳng đứng, không bị trượt đổ nghiêng (hiện tượng ngồi trượt mông ra trước). Xương chậu được ví như móng nhà trong cơ thể, khi xương chậu bị đổ nghiêng sẽ gây ra biến dạng cột sống, tăng sức ép trên đĩa đệm gây thoát vị đĩa đệm.&lt;/p&gt;
+&lt;p&gt;-Thiết kế lồi ở phần lưng, lõm ở phần mông và phần lồi ở mặt ghế tạo ra khối cấu trúc LOCK – HOLD ÔM CHẶT – GIỮ CHUẨN – CHỐNG TRƯỢT.&lt;/p&gt;
+&lt;p&gt;-Kích thước mặt ghế là 35cm, ngắn hơn ghế thông thường: đây là một điểm khác biệt có ưu thế giúp áp chặt lưng vào khối ÔM CHẶT – GIỮ CHUẢN – CHỐNG TRƯỢT. Thích hợp với chiều cao khác nhau của nhiều người, giúp hai chân đặt vững trên mặt đất.&lt;/p&gt;
+&lt;p&gt;TÁC DỤNG SẢN PHẨM&lt;/p&gt;
+&lt;p&gt;-Dùng để ngồi làm việc, học tập, sinh hoạt hàng ngày. Đồng thời có tác dụng ĐIỀU CHỈNH XƯƠNG CHẬU, XƯƠNG CÙNG, XƯƠNG SỐNG VỀ HÌNH DẠNG BÌNH THƯỜNG.&lt;/p&gt;
+&lt;p&gt;-Hiệu quả khi sử dụng: Phòng ngừa LỆCH VẸO và các bệnh cột sống phát sinh do ngồi sai tư thế.&lt;/p&gt;
+&lt;p&gt;-Ghế ngồi sáng chế DOCTORLOAN N85 cần thiết cho mọi người, mọi lúc, mọi nơi, trong sinh hoạt hằng ngày nhằm phòng ngừa bệnh cột sống do ngồi sai tư thế.&lt;/p&gt;
+&lt;p&gt;-Sản phẩm phù hợp sử dụng ở mọi nơi như trong gia đình, bệnh viện, phòng khám, trường học, sân bay, văn phòng làm việc và ngoài trời (sân vận động, trạm xe buýt, ).&lt;/p&gt;
+&lt;p&gt;CHẤT LIỆU:&lt;/p&gt;
+&lt;p&gt;-Nhựa PP nguyên sinh 100%&lt;/p&gt;
+&lt;p&gt;-Khả năng chịu lực lên đến 150 kg&lt;/p&gt;
+&lt;p&gt;BẢO HÀNH:&lt;/p&gt;
+&lt;p&gt;-Chân ghế: 3 năm&lt;/p&gt;
+&lt;p&gt;-Thân ghế: 3 năm&lt;/p&gt;
+&lt;p&gt;-Màu sắc: 1 năm theo tiêu chuẩn nhà sản xuất CÁCH CHỌN CHÂN GHẾ N85 – Ghế chân ngắn: dành cho người cao 1m45-1m75 ngồi với bàn 75cm. Nếu cao dưới 1m45 cần có bàn nâng hạ chiều cao&lt;/p&gt;
+&lt;p&gt;– Ghế chân dài: dành cho người cao trên 1m75 và cao dưới 1m45 ngồi với bàn cố định 75cm.&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="K9" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr"/>
+      <c r="M9" s="2" t="inlineStr"/>
+      <c r="N9" s="2" t="inlineStr"/>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768818009691-285486739-ghe-doctorloan-N85-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768818012323-28385882-ghe-doctorloan-N85-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768818014879-728436465-ghe-doctorloan-N85-4-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768818017040-468194579-ghe-doctorloan-N85-5-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768818019761-260275311-ghe-doctorloan-N85-6-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr"/>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ghe-doctorloan-90t</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế DoctorLoan 90T (Đệm Mỏng)</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>19699000</v>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767625421018-411885121-ghe-doctorloan-90T-1-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr"/>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/ghe-sang-che-doctorloan-90t-dem-mong/</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dựa trên mô phỏng đường cong cột sống sống, ghế sáng chế DOCTORLOAN 90T được thiết kế với cấu trúc đặc biệt “LỒI TRƯỚC – LÕM SAU” tạo nên chức năng “ÔM CHẶT – GIỮ CHUẨN – CHỐNG TRƯỢT”. Lõi ghế làm từ chất liệu composite (sợi thuỷ tinh) dùng đóng vỏ tảu, máy bay nên siêu cứng giúp tạo ra lực phản hồi mang đến khả năng tự điều chỉnh cột sống dưới tác động của trọng lực cơ thể. Tạo giải pháp tối ưu để duy trì đường cong sinh lý cột sống lưng, xương cùng cụt, giữ xương chậu ở tư thế thẳng và cân đối, bảo vệ cột sống trong tình trạng tốt nhất.&lt;/p&gt;
+&lt;p&gt;THIẾT KẾ&lt;/p&gt;
+&lt;p&gt;“Vùng gờ thắt lưng” giúp nâng đỡ và tạo lực đẩy giúp cho cột sống có độ cong tự nhiên giảm áp lực trên đĩa đệm. Đồng thời lõi cứng giúp tạo lực phản hồi để nắn chỉnh các đốt sống trật/ trượt về vị trí đúng, nắn chỉnh tạo hình đường cong sinh lý tự nhiên của cột sống lưng.&lt;/p&gt;
+&lt;p&gt;“Vùng hõm mặt ghế” giúp giữ vững cân đối khung chậu và xương cùng ở tư thế ngay ngắn khi ngồi. Đồng thời nắn chỉnh xương cùng cụt, cải thiện hiệu quả với tình trạng thoát vị đĩa đệm L5/S1 và thần kinh toạ.&lt;/p&gt;
+&lt;p&gt;“Vùng gờ lồi trung tâm” giúp chống trượt mông khi ngồi. Đồng thời giữ cho xương chậu luôn được thẳng đứng. Xương chậu được ví như móng nhà. Khi xương chậu thẳng sẽ giúp giữ chuẩn toàn bộ cấu trúc cột sống bên trên.&lt;/p&gt;
+&lt;p&gt;Ghế ngồi sáng chế DOCTORLOAN 90T giống như một khuôn ép sử dụng chính lực ép do trọng lượng cơ thể sinh ra để tác động lên toàn bộ khung xương cột sống, giữ chuẩn và điều chỉnh các chi tiết trượt/ trật về cấu trúc cân xứng.&lt;/p&gt;
+&lt;p&gt;• CÔNG DỤNG: Giúp giảm nhanh các triệu chứng&lt;/p&gt;
+&lt;p&gt;– Đau cấp tính thắt lưng, mông, chân khi vận động sai tư thế&lt;/p&gt;
+&lt;p&gt;– Đau lưng dữ dội hoặc âm ỉ kéo dài do: đau thần kinh toạ, đau thoát vị đĩa đệm cột sống lưng, trật vẹo cột sống thắt lưng&lt;/p&gt;
+&lt;p&gt;– Đau/ nhói ngực, khó thở do biến đổi cấu trúc cột sống ngực&lt;/p&gt;
+&lt;p&gt;– Đau do xương chậu và xương cùng bị biến dạng do nằm sai tư thế trong sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p&gt;– Tê / buốt/ mất cảm giác chân, ngón chân Hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cho mọi lứa tuổi&lt;/p&gt;
+&lt;p&gt;– Gù lưng – Thoát vị đĩa đệm – Thoái hóa cột sống&lt;/p&gt;
+&lt;p&gt;– Cong vẹo cột sống&lt;/p&gt;
+&lt;p&gt;– Trượt đốt sống&lt;/p&gt;
+&lt;p&gt;– Liệt tay, chân Hỗ trợ trong các trường hợp cột sống thắt lưng bị biến dạng, đang ở giai đoạn tiền phẫu hoặc hậu phẫu thuật&lt;/p&gt;
+&lt;p&gt;• ĐỐI TƯỢNG SỬ DỤNG: Ghế sáng chế 90D phù hợp với tất cả mọi người, ưu tiên để ngồi làm việc văn phòng, máy tính, viết, ngồi nghỉ ngơi, thư giãn, đọc sách, xem tivi.&lt;/p&gt;
+&lt;p&gt;CHẤT LIỆU&lt;/p&gt;
+&lt;p&gt;– Vỏ ghế được bọc bởi da Simili&lt;/p&gt;
+&lt;p&gt;– Lõi ghế làm từ Composite&lt;/p&gt;
+&lt;p&gt;– Chân ghế cấu tạo từ hợp kim nhôm&lt;/p&gt;
+&lt;p&gt;– Khả năng chịu lực lên đến 150kg&lt;/p&gt;
+&lt;p&gt;• KÍCH THƯỚC: – Dài – rộng – cao: 50 x 46 x [103-108] (cm)&lt;/p&gt;
+&lt;p&gt;– Khối lượng: 8,5 kg&lt;/p&gt;
+&lt;p&gt;• BẢO HÀNH:&lt;/p&gt;
+&lt;p&gt;– Phôi ghế Composite: 10 năm&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc Simili: 6 tháng&lt;/p&gt;
+&lt;p&gt;– Ben ghế/ mâm ống: 6 tháng&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="K10" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
+      <c r="N10" s="2" t="inlineStr"/>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768140223955-98262924-ghe-doctorloan-90T-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140227095-167738158-ghe-doctorloan-90T-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140237216-700907529-ghe-doctorloan-90T-4-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140240481-443563212-ghe-doctorloan-90T-5-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140243895-443544352-ghe-doctorloan-90T-6-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr"/>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>ghe-doctorloan-90d</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế DoctorLoan 90D (Đệm Dày)</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>34937000</v>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767625347313-807103995-ghe-doctorloan-90D-1-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr"/>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/4469/</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dựa trên mô phỏng đường cong cột sống sống, ghế sáng chế DOCTORLOAN 90D được thiết kế với cấu trúc “LỐI TRƯỚC – LÕM SAU” tạo nên chức năng “ÔM CHẶT – GIỮ CHUẨN – CHỐNG TRƯỢT”. Lõi ghế làm từ chất liệu composite (sợi thuỷ tinh) dùng đóng vỏ tảu, máy bay nên siêu cứng giúp tạo ra lực phản hồi mang đến khả năng tự điều chỉnh cột sống dưới tác động của trọng lực cơ thể. Tạo giải pháp tối ưu để duy trì đường cong sinh lý cột sống lưng, xương cùng cụt, giữ xương chậu ở tư thế thẳng và cân đối, bảo vệ cột sống trong tình trạng tốt nhất.&lt;/p&gt;
+&lt;p&gt;THIẾT KẾ&lt;/p&gt;
+&lt;p&gt;“Vùng gờ thắt lưng” giúp nâng đỡ và tạo lực đẩy giúp cho cột sống có độ cong tự nhiên giảm áp lực trên đĩa đệm. Đồng thời lõi cứng giúp tạo lực phản hồi để nắn chỉnh các đốt sống trật/ trượt về vị trí đúng, nắn chỉnh tạo hình đường cong sinh lý tự nhiên của cột sống lưng.&lt;/p&gt;
+&lt;p&gt;“Vùng hõm mặt ghế” giúp giữ vững cân đối khung chậu và xương cùng ở tư thế ngay ngắn khi ngồi. Đồng thời nắn chỉnh xương cùng cụt, cải thiện hiệu quả với tình trạng thoát vị đĩa đệm L5/S1 và thần kinh toạ.&lt;/p&gt;
+&lt;p&gt;“Vùng gờ lồi trung tâm” giúp chống trượt mông khi ngồi. Đồng thời giữ cho xương chậu luôn được thẳng đứng. Xương chậu được ví như móng nhà. Khi xương chậu thẳng sẽ giúp giữ chuẩn toàn bộ cấu trúc cột sống bên trên.&lt;/p&gt;
+&lt;p&gt;Ghế ngồi sáng chế DOCTORLOAN 90T giống như một khuôn ép sử dụng chính lực ép do trọng lượng cơ thể sinh ra để tác động lên toàn bộ khung xương cột sống, giữ chuẩn và điều chỉnh các chi tiết trượt/ trật về cấu trúc cân xứng.&lt;/p&gt;
+&lt;p&gt;• CÔNG DỤNG: Giúp giảm nhanh các triệu chứng&lt;/p&gt;
+&lt;p&gt;– Đau cấp tính thắt lưng, mông, chân khi vận động sai tư thế&lt;/p&gt;
+&lt;p&gt;– Đau lưng dữ dội hoặc âm ỉ kéo dài do: đau thần kinh toạ, đau thoát vị đĩa đệm cột sống lưng, trật vẹo cột sống thắt lưng&lt;/p&gt;
+&lt;p&gt;– Đau/ nhói ngực, khó thở do biến đổi cấu trúc cột sống ngực&lt;/p&gt;
+&lt;p&gt;– Đau do xương chậu và xương cùng bị biến dạng do nằm sai tư thế trong sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p&gt;– Tê / buốt/ mất cảm giác chân, ngón chân Hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cho mọi lứa tuổi&lt;/p&gt;
+&lt;p&gt;– Gù lưng – Thoát vị đĩa đệm – Thoái hóa cột sống&lt;/p&gt;
+&lt;p&gt;– Cong vẹo cột sống&lt;/p&gt;
+&lt;p&gt;– Trượt đốt sống&lt;/p&gt;
+&lt;p&gt;– Liệt tay, chân Hỗ trợ trong các trường hợp cột sống thắt lưng bị biến dạng, đang ở giai đoạn tiền phẫu hoặc hậu phẫu thuật&lt;/p&gt;
+&lt;p&gt;• ĐỐI TƯỢNG SỬ DỤNG: Ghế sáng chế 90D phù hợp với tất cả mọi người, ưu tiên để ngồi làm việc văn phòng, máy tính, viết, ngồi nghỉ ngơi, thư giãn, đọc sách, xem tivi.&lt;/p&gt;
+&lt;p&gt;CHẤT LIỆU&lt;/p&gt;
+&lt;p&gt;– Vỏ ghế được bọc bởi da Simili&lt;/p&gt;
+&lt;p&gt;– Lõi ghế làm từ Composite&lt;/p&gt;
+&lt;p&gt;– Chân ghế cấu tạo từ hợp kim nhôm&lt;/p&gt;
+&lt;p&gt;– Khả năng chịu lực lên đến 150kg&lt;/p&gt;
+&lt;p&gt;• KÍCH THƯỚC: – Dài – rộng – cao: 50 x 46 x [103-108] (cm)&lt;/p&gt;
+&lt;p&gt;– Khối lượng: 8,5 kg&lt;/p&gt;
+&lt;p&gt;• BẢO HÀNH:&lt;/p&gt;
+&lt;p&gt;– Phôi ghế Composite: 10 năm&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc Simili: 6 tháng&lt;/p&gt;
+&lt;p&gt;– Ben ghế/ mâm ống: 6 tháng&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>10</v>
+      </c>
+      <c r="K11" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr"/>
+      <c r="M11" s="2" t="inlineStr"/>
+      <c r="N11" s="2" t="inlineStr"/>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768140309895-247593817-ghe-doctorloan-90D-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140312983-105642804-ghe-doctorloan-90D-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140315535-147315026-ghe-doctorloan-90D-4-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140318449-902680379-ghe-doctorloan-90D-5-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140320747-389093713-ghe-doctorloan-90D-6-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr"/>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>ghe-doctorloan-95</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế DoctorLoan 95</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>39249000</v>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767625245640-463910034-ghe-doctorloan-95-1-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr"/>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/ghe-sang-che-doctorloan-95/</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dựa trên mô phỏng đường cong cột sống sống, ghế sáng chế DOCTORLOAN 95 được thiết kế với cấu trúc “LỒI TRƯỚC – LÕM SAU” tạo nên chức năng “ÔM CHẶT – GIỮ CHUẨN – CHỐNG TRƯỢT”. Lõi ghế làm từ chất liệu composite (sợi thuỷ tinh) dùng đóng vỏ tảu, máy bay nên siêu cứng giúp tạo ra lực phản hồi mang đến khả năng tự điều chỉnh cột sống dưới tác động của trọng lực cơ thể. Tạo giải pháp tối ưu để duy trì đường cong sinh lý cột sống lưng, xương cùng cụt, giữ xương chậu ở tư thế thẳng và cân đối, bảo vệ cột sống trong tình trạng tốt nhất.&lt;/p&gt;
+&lt;p&gt;THIẾT KẾ&lt;/p&gt;
+&lt;p&gt;“Vùng gờ thắt lưng” giúp nâng đỡ và tạo lực đẩy giúp cho cột sống có độ cong tự nhiên giảm áp lực trên đĩa đệm. Đồng thời lõi cứng giúp tạo lực phản hồi để nắn chỉnh các đốt sống trật/ trượt về vị trí đúng, nắn chỉnh tạo hình đường cong sinh lý tự nhiên của cột sống lưng.&lt;/p&gt;
+&lt;p&gt;“Vùng hõm mặt ghế” giúp giữ vững cân đối khung chậu và xương cùng ở tư thế ngay ngắn khi ngồi. Đồng thời nắn chỉnh xương cùng cụt, cải thiện hiệu quả với tình trạng thoát vị đĩa đệm L5/S1 và thần kinh toạ.&lt;/p&gt;
+&lt;p&gt;“Vùng gờ lồi trung tâm” giúp chống trượt mông khi ngồi. Đồng thời giữ cho xương chậu luôn được thẳng đứng. Xương chậu được ví như móng nhà. Khi xương chậu thẳng sẽ giúp giữ chuẩn toàn bộ cấu trúc cột sống bên trên.&lt;/p&gt;
+&lt;p&gt;Ghế ngồi sáng chế DOCTORLOAN 90T giống như một khuôn ép sử dụng chính lực ép do trọng lượng cơ thể sinh ra để tác động lên toàn bộ khung xương cột sống, giữ chuẩn và điều chỉnh các chi tiết trượt/ trật về cấu trúc cân xứng.&lt;/p&gt;
+&lt;p&gt;• CÔNG DỤNG: Giúp giảm nhanh các triệu chứng&lt;/p&gt;
+&lt;p&gt;– Đau cấp tính thắt lưng, mông, chân khi vận động sai tư thế&lt;/p&gt;
+&lt;p&gt;– Đau lưng dữ dội hoặc âm ỉ kéo dài do: đau thần kinh toạ, đau thoát vị đĩa đệm cột sống lưng, trật vẹo cột sống thắt lưng&lt;/p&gt;
+&lt;p&gt;– Đau/ nhói ngực, khó thở do biến đổi cấu trúc cột sống ngực&lt;/p&gt;
+&lt;p&gt;– Đau do xương chậu và xương cùng bị biến dạng do nằm sai tư thế trong sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p&gt;– Tê / buốt/ mất cảm giác chân, ngón chân Hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cho mọi lứa tuổi&lt;/p&gt;
+&lt;p&gt;– Gù lưng – Thoát vị đĩa đệm – Thoái hóa cột sống&lt;/p&gt;
+&lt;p&gt;– Cong vẹo cột sống&lt;/p&gt;
+&lt;p&gt;– Trượt đốt sống&lt;/p&gt;
+&lt;p&gt;– Liệt tay, chân Hỗ trợ trong các trường hợp cột sống thắt lưng bị biến dạng, đang ở giai đoạn tiền phẫu hoặc hậu phẫu thuật&lt;/p&gt;
+&lt;p&gt;• ĐỐI TƯỢNG SỬ DỤNG: Ghế sáng chế 90D phù hợp với tất cả mọi người, ưu tiên để ngồi làm việc văn phòng, máy tính, viết, ngồi nghỉ ngơi, thư giãn, đọc sách, xem tivi.&lt;/p&gt;
+&lt;p&gt;CHẤT LIỆU&lt;/p&gt;
+&lt;p&gt;– Vỏ ghế được bọc bởi da Simili&lt;/p&gt;
+&lt;p&gt;– Lõi ghế làm từ Composite&lt;/p&gt;
+&lt;p&gt;– Chân ghế cấu tạo từ hợp kim nhôm&lt;/p&gt;
+&lt;p&gt;– Khả năng chịu lực lên đến 150kg&lt;/p&gt;
+&lt;p&gt;• KÍCH THƯỚC: – Dài – rộng – cao: 50 x 46 x [103-108] (cm)&lt;/p&gt;
+&lt;p&gt;– Khối lượng: 8,5 kg&lt;/p&gt;
+&lt;p&gt;• BẢO HÀNH:&lt;/p&gt;
+&lt;p&gt;– Phôi ghế Composite: 10 năm&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc Simili: 6 tháng&lt;/p&gt;
+&lt;p&gt;– Ben ghế/ mâm ống: 6 tháng&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr"/>
+      <c r="M12" s="2" t="inlineStr"/>
+      <c r="N12" s="2" t="inlineStr"/>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1769510059222-392818248-ghe-doctorloan-95-2-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1769510062134-944276652-ghe-doctorloan-95-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1769510064920-292094931-ghe-doctorloan-95-4-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1769510067303-500229386-ghe-doctorloan-95-5-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1769510069675-267535634-ghe-doctorloan-95-6-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr"/>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>ghe-doctorloan-135</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế DoctorLoan 135</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>53762000</v>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767625106166-637783990-ghe-doctorloan-135-1-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr"/>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/ghe-sang-che-doctorloan-135/</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dựa trên mô phỏng đường cong cột sống sống, ghế sáng chế DOCTORLOAN 150 được thiết kế với phần lồi phía trước, lõm phía sau và gờ lồi trung tâm tạo nên chức năng “ÔM CHẶT – GIỮ CHUẨN – CHỐNG TRƯỢT”. Lõi ghế làm từ chất liệu composite (sợi thuỷ tinh) dùng đóng vỏ tảu, máy bay nên siêu cứng giúp tạo ra lực phản hồi mang đến khả năng tự điều chỉnh cột sống dưới tác động của trọng lực cơ thể. Tạo giải pháp tối ưu để duy trì đường cong sinh lý cột sống cổ, ngực, lưng, xương cùng cụt và xương chậu. Giúp bảo vệ cột sống trong tình trạng tốt nhất.&lt;/p&gt;
+&lt;p&gt;THIẾT KẾ:&lt;/p&gt;
+&lt;p&gt;Ghế sáng chế DOCTORLOAN 150 được thiết kế đặc biệt với độ ngả 150˚, kết hợp với các đường cong LỒI TRƯỚC LÕM SAU uốn theo cấu trúc cong tự nhiên của cột sống giúp giảm sâu áp lực trên cột sống, đĩa đệm, khung xương. Đồng thời giúp nắn chỉnh các sai lệch đốt sống, tạo hình lại đường cong sinh lý. “Vùng đầu” lồi ra trước giúp nâng đỡ và nắn chỉnh Cột Sống Cổ ” Vùng ngực” lõm ra sau đúng theo cấu trúc cột sống ngực “Vùng gờ thắt lưng” giúp nâng đỡ và tạo lực đẩy giúp cho cột sống có độ cong tự nhiên giảm áp lực trên đĩa đệm. Đồng thời lõi cứng giúp tạo lực phản hồi để nắn chỉnh các đốt sống trật/ trượt về vị trí đúng, nắn chỉnh tạo hình đường cong sinh lý tự nhiên của cột sống lưng. “Vùng hõm mặt ghế” giúp giữ chuẩn cấu trúc khung chậu và xương cùng cụt ở tư thế ngay ngắn khi nằm. “Gờ lồi trung tâm” giúp chống trượt mông khi nằm.&lt;/p&gt;
+&lt;p&gt;CÔNG DỤNG: Giúp giảm nhanh các triệu chứng&lt;/p&gt;
+&lt;p&gt;– Đau cấp tính thắt lưng, mông, chân khi vận động sai tư thế&lt;/p&gt;
+&lt;p&gt;– Đau lưng dữ dội hoặc âm ỉ kéo dài do: đau thần kinh toạ, đau thoát vị đĩa đệm cột sống lưng, trật vẹo cột sống thắt lưng&lt;/p&gt;
+&lt;p&gt;– Đau/ nhói ngực, khó thở do biến đổi cấu trúc cột sống ngực&lt;/p&gt;
+&lt;p&gt;– Đau do xương chậu và xương cùng bị biến dạng do nằm sai tư thế trong sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p&gt;– Tê / buốt/ mất cảm giác chân, ngón chân&lt;/p&gt;
+&lt;p&gt;Hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cho mọi lứa tuổi&lt;/p&gt;
+&lt;p&gt;– Gù lưng&lt;/p&gt;
+&lt;p&gt;– Thoát vị đĩa đệm&lt;/p&gt;
+&lt;p&gt;– Thoái hóa cột sống&lt;/p&gt;
+&lt;p&gt;– Cong vẹo cột sống&lt;/p&gt;
+&lt;p&gt;– Trượt đốt sống&lt;/p&gt;
+&lt;p&gt;– Liệt tay, chân&lt;/p&gt;
+&lt;p&gt;– Hỗ trợ trong các trường hợp cột sống thắt lưng bị biến dạng, đang ở giai đoạn tiền phẫu hoặc hậu phẫu thuật&lt;/p&gt;
+&lt;p&gt;• ĐỐI TƯỢNG SỬ DỤNG: Ghế sáng chế 150 phù hợp nằm nghỉ ngơi, thư giãn, đọc sách, xem tivi và ngủ trưa. Cả gia đình có thể cùng sử dụng&lt;/p&gt;
+&lt;p&gt;• CHẤT LIỆU&lt;/p&gt;
+&lt;p&gt;– Phôi ghế làm từ Composite, bọc Da smili&lt;/p&gt;
+&lt;p&gt;– Phần đệm mặt ghế &amp; lưng ghế được cấu tạo từ mút&lt;/p&gt;
+&lt;p&gt;– Chân ghế làm từ Inox 304 – Tay vịn ghế: bên trong làm bằng gỗ được bọc Da simili&lt;/p&gt;
+&lt;p&gt;– Đôn ghế: ruột đôn ghế bằng mút được bọc Da simili&lt;/p&gt;
+&lt;p&gt;– Khả năng chịu lực lên đến 200kg&lt;/p&gt;
+&lt;p&gt;• KÍCH THƯỚC&lt;/p&gt;
+&lt;p&gt;– Dài x rộng x cao: 143 x 68 x 102 (cm)&lt;/p&gt;
+&lt;p&gt;– Khối lượng: 17,8 kg&lt;/p&gt;
+&lt;p&gt;• BẢO HÀNH:&lt;/p&gt;
+&lt;p&gt;– Phôi ghế Composite: 10 năm&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc Simili: 6 tháng&lt;/p&gt;
+&lt;p&gt;– Chân ghế/ ben ghế/ mâm ống: 6 tháng&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>12</v>
+      </c>
+      <c r="K13" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr"/>
+      <c r="M13" s="2" t="inlineStr"/>
+      <c r="N13" s="2" t="inlineStr"/>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768140346486-368327387-ghe-doctorloan-135-5-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140344247-642771782-ghe-doctorloan-135-4-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140341927-915795478-ghe-doctorloan-135-3-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140348679-896385088-ghe-doctorloan-135-6-scaled.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1768140338441-797966276-ghe-doctorloan-135-2-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr"/>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ghe-doctorloan-150</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế DoctorLoan 150</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="n">
+        <v>53762000</v>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1767625218826-745244216-z571322856284909e27ff18e338012c913dff5f1193f0f.jpg</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr"/>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/ghe-sang-che-doctorloan-150/</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dựa trên mô phỏng đường cong cột sống sống, ghế sáng chế DOCTORLOAN 150 được thiết kế với phần lồi phía trước, lõm phía sau và gờ lồi trung tâm tạo nên chức năng “ÔM CHẶT – GIỮ CHUẨN – CHỐNG TRƯỢT”. Lõi ghế làm từ chất liệu composite (sợi thuỷ tinh) dùng đóng vỏ tảu, máy bay nên siêu cứng giúp tạo ra lực phản hồi mang đến khả năng tự điều chỉnh cột sống dưới tác động của trọng lực cơ thể. Tạo giải pháp tối ưu để duy trì đường cong sinh lý cột sống cổ, ngực, lưng, xương cùng cụt và xương chậu. Giúp bảo vệ cột sống trong tình trạng tốt nhất.&lt;/p&gt;
+&lt;p&gt;THIẾT KẾ:&lt;/p&gt;
+&lt;p&gt;Ghế sáng chế DOCTORLOAN 150 được thiết kế đặc biệt với độ ngả 150˚, kết hợp với các đường cong LỒI TRƯỚC LÕM SAU uốn theo cấu trúc cong tự nhiên của cột sống giúp giảm sâu áp lực trên cột sống, đĩa đệm, khung xương. Đồng thời giúp nắn chỉnh các sai lệch đốt sống, tạo hình lại đường cong sinh lý. “Vùng đầu” lồi ra trước giúp nâng đỡ và nắn chỉnh Cột Sống Cổ ” Vùng ngực” lõm ra sau đúng theo cấu trúc cột sống ngực “Vùng gờ thắt lưng” giúp nâng đỡ và tạo lực đẩy giúp cho cột sống có độ cong tự nhiên giảm áp lực trên đĩa đệm. Đồng thời lõi cứng giúp tạo lực phản hồi để nắn chỉnh các đốt sống trật/ trượt về vị trí đúng, nắn chỉnh tạo hình đường cong sinh lý tự nhiên của cột sống lưng. “Vùng hõm mặt ghế” giúp giữ chuẩn cấu trúc khung chậu và xương cùng cụt ở tư thế ngay ngắn khi nằm. “Gờ lồi trung tâm” giúp chống trượt mông khi nằm.&lt;/p&gt;
+&lt;p&gt;CÔNG DỤNG: Giúp giảm nhanh các triệu chứng&lt;/p&gt;
+&lt;p&gt;– Đau cấp tính thắt lưng, mông, chân khi vận động sai tư thế&lt;/p&gt;
+&lt;p&gt;– Đau lưng dữ dội hoặc âm ỉ kéo dài do: đau thần kinh toạ, đau thoát vị đĩa đệm cột sống lưng, trật vẹo cột sống thắt lưng&lt;/p&gt;
+&lt;p&gt;– Đau/ nhói ngực, khó thở do biến đổi cấu trúc cột sống ngực&lt;/p&gt;
+&lt;p&gt;– Đau do xương chậu và xương cùng bị biến dạng do nằm sai tư thế trong sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p&gt;– Tê / buốt/ mất cảm giác chân, ngón chân&lt;/p&gt;
+&lt;p&gt;Hỗ trợ điều trị và ngăn ngừa các bệnh cột sống cho mọi lứa tuổi&lt;/p&gt;
+&lt;p&gt;– Gù lưng&lt;/p&gt;
+&lt;p&gt;– Thoát vị đĩa đệm&lt;/p&gt;
+&lt;p&gt;– Thoái hóa cột sống&lt;/p&gt;
+&lt;p&gt;– Cong vẹo cột sống&lt;/p&gt;
+&lt;p&gt;– Trượt đốt sống&lt;/p&gt;
+&lt;p&gt;– Liệt tay, chân&lt;/p&gt;
+&lt;p&gt;– Hỗ trợ trong các trường hợp cột sống thắt lưng bị biến dạng, đang ở giai đoạn tiền phẫu hoặc hậu phẫu thuật&lt;/p&gt;
+&lt;p&gt;• ĐỐI TƯỢNG SỬ DỤNG: Ghế sáng chế 150 phù hợp nằm nghỉ ngơi, thư giãn, đọc sách, xem tivi và ngủ trưa. Cả gia đình có thể cùng sử dụng&lt;/p&gt;
+&lt;p&gt;• CHẤT LIỆU&lt;/p&gt;
+&lt;p&gt;– Phôi ghế làm từ Composite, bọc Da smili&lt;/p&gt;
+&lt;p&gt;– Phần đệm mặt ghế &amp; lưng ghế được cấu tạo từ mút&lt;/p&gt;
+&lt;p&gt;– Chân ghế làm từ Inox 304 – Tay vịn ghế: bên trong làm bằng gỗ được bọc Da simili&lt;/p&gt;
+&lt;p&gt;– Đôn ghế: ruột đôn ghế bằng mút được bọc Da simili&lt;/p&gt;
+&lt;p&gt;– Khả năng chịu lực lên đến 200kg&lt;/p&gt;
+&lt;p&gt;• KÍCH THƯỚC&lt;/p&gt;
+&lt;p&gt;– Dài x rộng x cao: 143 x 68 x 102 (cm)&lt;/p&gt;
+&lt;p&gt;– Khối lượng: 17,8 kg&lt;/p&gt;
+&lt;p&gt;• BẢO HÀNH:&lt;/p&gt;
+&lt;p&gt;– Phôi ghế Composite: 10 năm&lt;/p&gt;
+&lt;p&gt;– Vỏ bọc Simili: 6 tháng&lt;/p&gt;
+&lt;p&gt;– Chân ghế/ ben ghế/ mâm ống: 6 tháng&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J14" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="K14" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr"/>
+      <c r="M14" s="2" t="inlineStr"/>
+      <c r="N14" s="2" t="inlineStr"/>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>Ghế sáng chế</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1769510102794-214988345-z571322856776408a8de1a8c2640793c3bb97a929f5780.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1769510107425-363350771-z5713228576163eb7d3123f64d26ea0788d28a003c9fc7.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1769510110677-460947288-z5713228579373c4d4cd3066f4066b2d42f42a26ecd1e9copy.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1769510115069-219723353-z5713228587328ea7a48cdd76df79780935f33e3ed8140.jpg
+https://hongcotsong.com/wp-content/uploads/2024/08/1769510122156-203832683-z5713228589452e6721a95f346077fd1d0ef8d40d965d3.jpg</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr"/>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>dem-doctorloan</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Đệm sáng chế DoctorLoan</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="n">
+        <v>6000000</v>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768818488781-178345811-dem-doctorloan-0-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr"/>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/dem-sang-che-doctorloan/</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;ĐẶC ĐIỂM CỦA SẢN PHẨM&lt;/p&gt;
+&lt;p&gt;Đây là sản phẩm có công dụng hỗ trợ điều trị và ngăn ngừa các bệnh cột sống lưng, giúp cột sống khỏe mạnh. Giữ cho xương chậu được thẳng và cấu trúc cột sống bình thường khi ngồi trên sàn. Điều chỉnh trật, lệch, vẹo của xương cùng khung chậu về cấu trúc bình thường&lt;/p&gt;
+&lt;p&gt;KIỂU DÁNG VÀ Ý TƯỞNG&lt;/p&gt;
+&lt;p&gt;Đệm ngồi được thiết kế với các bậc uốn cong theo cấu trúc xương chậu – xương cùng – xương cụt. Đệm ngồi sáng chế DOCTORLOAN – giải pháp chăm sóc khung xương chậu và xương sống an toàn và hiệu quả. Sử dụng công nghệ sáng chế vượt trội tạo kết cấu đặc biệt (đã được bảo hộ độc quyền).&lt;br /&gt;
+CHẤT LIỆU&lt;/p&gt;
+&lt;p&gt;– Ruột đệm làm từ mút PU FOAM có tỷ trọng cao, độ bền tốt được kiểm định chất lượng, độ an toàn tại cơ quan kiểm định chất lượng TP Hồ Chí Minh. – Phần lõi được làm từ chất liệu EPS siêu cứng có khả năng chịu lực rất tốt – Vỏ bọc da Simili cao cấp tạo độ sang trọng và được kiểm định về chất lượng&lt;/p&gt;
+&lt;p&gt;ỨNG DỤNG&lt;/p&gt;
+&lt;p&gt;– Giữ cho xương chậu được thẳng và cấu trúc cột sống bình thường khi ngồi trên sàn – Phòng và điều chỉnh trật, lệch, vẹo của xương cùng, khung xương chậu do thói quen ngồi bệt dưới sàn về cấu trúc bình thường – Nhanh chóng giảm áp lực lên đĩa đệm và cột sống. Hết đau đầu gối, đau mông khi ngồi trên sàn – Thích hợp dùng làm đệm ngồi bệt, nệm ngồi bàn thấp, nệm ngồi trà đạo, nệm ngồi bàn trà kiểu Nhật, nệm lót ngồi thiền, ngồi thư giãn, hay nệm lót ngồi trang trí trên ghế tựa, ghế mây, ghế gỗ.&lt;/p&gt;
+&lt;p&gt;BẢO HÀNH:&lt;/p&gt;
+&lt;p&gt;– Ruột đệm: bảo hành 01 tháng&lt;/p&gt;
+&lt;p&gt;– Lõi đệm: bảo hành 01 năm&lt;/p&gt;
+&lt;p&gt;– Vỏ đệm simili: bảo hành 06 tháng&lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J15" s="2" t="n">
+        <v>14</v>
+      </c>
+      <c r="K15" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
+      <c r="N15" s="2" t="inlineStr"/>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>Đệm sáng chế</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768818496310-801838474-dem-doctorloan-2-scaled.jpg</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr"/>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>combo-co-ban-1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>COMBO Nắn Chỉnh Cơ Bản 1</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="n">
+        <v>8307000</v>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768833282105-976548564-Combocoban3.webp</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr"/>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/combo-co-ban-1/</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Bảo vệ cơ bản cột sống với giải pháp DoctorLoan – Gối sáng chế DoctorLoan: Nắn chỉnh chuyên sâu cột sống cổ và cột sống lưng – Ghế sáng chế DoctorLoan N85: Giữ dáng ngồi chuẩn trong các sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;strong&gt;DoctorLoan&lt;/strong&gt; mang đến giải pháp hỗ trợ tư thế và chăm sóc cột sống thông qua các sản phẩm được thiết kế chuyên biệt, giúp người dùng chủ động bảo vệ cột sống trong sinh hoạt hằng ngày.&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;Gối sáng chế DoctorLoan&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4945-2" aria-describedby="caption-attachment-4945-2" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4945 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1767577012969-211026264-goi-co-doctorloan-f4-2-1000x1000-1-800x800.jpg" alt="Gối sáng chế DoctorLoan" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4945-2" class="wp-caption-text"&gt;Gối sáng chế DoctorLoan&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;Hỗ trợ &lt;strong&gt;nắn chỉnh chuyên sâu cột sống cổ và cột sống lưng&lt;/strong&gt;, giúp định hướng tư thế phù hợp trong quá trình nghỉ ngơi và sinh hoạt.&lt;/p&gt;
+&lt;h3 class="product-title product_title entry-title"&gt;&lt;strong&gt;Gối lưng sáng chế DoctorLoan F4&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4944-2" aria-describedby="caption-attachment-4944-2" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4944 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140445042-521234568-goi-lung-doctorloan-f3-5-1000x1000-1-800x800.jpg" alt="Gối lưng sáng chế DoctorLoan F4" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4944-2" class="wp-caption-text"&gt;Gối lưng sáng chế DoctorLoan F4&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;div class="product-short-description"&gt;
+&lt;p&gt;Gối lưng sáng chế DoctorLoan F4 giúp bảo vệ và nắn chỉnh lại các sai lệch đốt sống lưng, ngực&lt;/p&gt;
+&lt;/div&gt;
+&lt;h3&gt;&lt;strong&gt;Ghế sáng chế DoctorLoan N85&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4950-4" aria-describedby="caption-attachment-4950-4" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4950 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140199100-761249413-ghe-doctorloan-N85-3-1000x1000-1-800x800.jpg" alt="Ghế sáng chế DoctorLoan N85 CHÂN NGẮN" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4950-4" class="wp-caption-text"&gt;Ghế sáng chế DoctorLoan N85 CHÂN NGẮN&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;Hỗ trợ &lt;strong&gt;duy trì dáng ngồi chuẩn trong các hoạt động hằng ngày&lt;/strong&gt;, góp phần hình thành thói quen ngồi khoa học và giảm áp lực không cần thiết lên cột sống.&lt;/p&gt;
+&lt;p&gt;DoctorLoan – đồng hành cùng bạn xây dựng tư thế khoa học và chủ động chăm sóc cột sống mỗi ngày.&lt;/p&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;SẢN PHẨM TRONG COMBO&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/goi-co-sang-che-doctorloan-f5/"&gt;– Gối cổ sáng chế DoctorLoan F5 : 4.312.000vnđ&lt;/a&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/goi-lung-sang-che-doctorloan-f1-goi-dai/"&gt;– Gối lưng sáng chế DoctorLoan F1 GỐI DÀI: 1.868.000vnđ&lt;/a&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/ghe-sang-che-doctorloan-n85-chan-ngan/"&gt;– Ghế sáng chế DoctorLoan N85 CHÂN NGẮN: 2.127.000 vnđ&lt;/a&gt;&lt;/h1&gt;</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J16" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="K16" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr"/>
+      <c r="M16" s="2" t="inlineStr"/>
+      <c r="N16" s="2" t="inlineStr"/>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>Gói Combo</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr"/>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr"/>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>combo-co-ban-2</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>COMBO Nắn Chỉnh Cơ Bản 2</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="n">
+        <v>12913000</v>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768833303409-131369072-Combocoban2.webp</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr"/>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/combo-co-ban-2/</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Bảo vệ cơ bản cột sống với giải pháp DoctorLoan – Gối sáng chế DoctorLoan: Nắn chỉnh chuyên sâu cột sống cổ và cột sống lưng – Ghế sáng chế DoctorLoan N85: Giữ dáng ngồi chuẩn trong các sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;strong&gt;DoctorLoan&lt;/strong&gt; mang đến giải pháp hỗ trợ tư thế và chăm sóc cột sống thông qua các sản phẩm được thiết kế chuyên biệt, giúp người dùng chủ động bảo vệ cột sống trong sinh hoạt hằng ngày.&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;Gối sáng chế DoctorLoan&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4845" aria-describedby="caption-attachment-4845" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4845 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2024/08/1768140488169-266575898-goi-co-doctorloan-f6-6-800x800.jpg" alt="Gối cổ sáng chế DoctorLoan F6" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4845" class="wp-caption-text"&gt;Gối cổ sáng chế DoctorLoan F6&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;Hỗ trợ &lt;strong&gt;nắn chỉnh chuyên sâu cột sống cổ và cột sống lưng&lt;/strong&gt;, giúp định hướng tư thế phù hợp trong quá trình nghỉ ngơi và sinh hoạt.&lt;/p&gt;
+&lt;h3 class="product-title product_title entry-title"&gt;&lt;strong&gt;Gối lưng sáng chế DoctorLoan F4&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4819-2" aria-describedby="caption-attachment-4819-2" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4819 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2024/08/1768140422559-802203686-goi-lung-doctorloan-f4-5-800x800.jpg" alt="Gối lưng sáng chế DoctorLoan F4" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4819-2" class="wp-caption-text"&gt;Gối lưng sáng chế DoctorLoan F4&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;div class="product-short-description"&gt;
+&lt;p&gt;Gối lưng sáng chế DoctorLoan F4 giúp bảo vệ và nắn chỉnh lại các sai lệch đốt sống lưng, ngực&lt;/p&gt;
+&lt;/div&gt;
+&lt;h3&gt;&lt;strong&gt;Ghế sáng chế DoctorLoan N85&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4950-3" aria-describedby="caption-attachment-4950-3" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4950 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140199100-761249413-ghe-doctorloan-N85-3-1000x1000-1-800x800.jpg" alt="Ghế sáng chế DoctorLoan N85 CHÂN NGẮN" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4950-3" class="wp-caption-text"&gt;Ghế sáng chế DoctorLoan N85 CHÂN NGẮN&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;Hỗ trợ &lt;strong&gt;duy trì dáng ngồi chuẩn trong các hoạt động hằng ngày&lt;/strong&gt;, góp phần hình thành thói quen ngồi khoa học và giảm áp lực không cần thiết lên cột sống.&lt;/p&gt;
+&lt;p&gt;DoctorLoan – đồng hành cùng bạn xây dựng tư thế khoa học và chủ động chăm sóc cột sống mỗi ngày.&lt;/p&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;
+SẢN PHẨM TRONG COMBO&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/goi-co-sang-che-doctorloan-f6/"&gt;– Gối cổ sáng chế DoctorLoan F6: 7.049.000 vnđ&lt;/a&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/goi-lung-sang-che-doctorloan-f4/"&gt;– Gối lưng sáng chế DoctorLoan F4: 3.737.000 vnđ&lt;/a&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/ghe-sang-che-doctorloan-n85-chan-ngan/"&gt;-Ghế sáng chế DoctorLoan N85 CHÂN NGẮN: 2.127.000 vnđ&lt;/a&gt;&lt;/h1&gt;
+&lt;p&gt; &lt;/p&gt;
+&lt;p&gt; &lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J17" s="2" t="n">
+        <v>16</v>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr"/>
+      <c r="M17" s="2" t="inlineStr"/>
+      <c r="N17" s="2" t="inlineStr"/>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>Gói Combo</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr"/>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr"/>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>combo-co-ban-3</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>COMBO Nắn Chỉnh Cơ Bản 3</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="n">
+        <v>13488000</v>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2024/08/1768833282105-976548564-Combocoban3-1.webp</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr"/>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/hang-gai-pho-4/</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Bảo vệ cơ bản cột sống với giải pháp DoctorLoan – Gối sáng chế DoctorLoan: Nắn chỉnh chuyên sâu cột sống cổ và cột sống lưng – Ghế sáng chế DoctorLoan N85: Giữ dáng ngồi chuẩn trong các sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;strong&gt;DoctorLoan&lt;/strong&gt; mang đến giải pháp hỗ trợ tư thế và chăm sóc cột sống thông qua các sản phẩm được thiết kế chuyên biệt, giúp người dùng chủ động bảo vệ cột sống trong sinh hoạt hằng ngày.&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;Gối sáng chế DoctorLoan F4&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4948-3" aria-describedby="caption-attachment-4948-3" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4948 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140497963-707220928-goi-co-doctorloan-f4-3-1000x1000-1-800x800.jpg" alt="Gối cổ sáng chế DoctorLoan F4" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4948-3" class="wp-caption-text"&gt;Gối cổ sáng chế DoctorLoan F4&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;Hỗ trợ &lt;strong&gt;nắn chỉnh chuyên sâu cột sống cổ và cột sống lưng&lt;/strong&gt;, giúp định hướng tư thế phù hợp trong quá trình nghỉ ngơi và sinh hoạt.&lt;/p&gt;
+&lt;h3 class="product-title product_title entry-title"&gt;&lt;strong&gt;Gối lưng sáng chế DoctorLoan F4&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4819" aria-describedby="caption-attachment-4819" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4819 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2024/08/1768140422559-802203686-goi-lung-doctorloan-f4-5-800x800.jpg" alt="Gối lưng sáng chế DoctorLoan F4" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4819" class="wp-caption-text"&gt;Gối lưng sáng chế DoctorLoan F4&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;div class="product-short-description"&gt;
+&lt;p&gt;Gối lưng sáng chế DoctorLoan F4 giúp bảo vệ và nắn chỉnh lại các sai lệch đốt sống lưng, ngực&lt;/p&gt;
+&lt;/div&gt;
+&lt;h3&gt;&lt;strong&gt;Ghế sáng chế DoctorLoan N85&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4950-2" aria-describedby="caption-attachment-4950-2" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4950 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140199100-761249413-ghe-doctorloan-N85-3-1000x1000-1-800x800.jpg" alt="Ghế sáng chế DoctorLoan N85 CHÂN NGẮN" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4950-2" class="wp-caption-text"&gt;Ghế sáng chế DoctorLoan N85 CHÂN NGẮN&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;Hỗ trợ &lt;strong&gt;duy trì dáng ngồi chuẩn trong các hoạt động hằng ngày&lt;/strong&gt;, góp phần hình thành thói quen ngồi khoa học và giảm áp lực không cần thiết lên cột sống.&lt;/p&gt;
+&lt;p&gt;DoctorLoan – đồng hành cùng bạn xây dựng tư thế khoa học và chủ động chăm sóc cột sống mỗi ngày.&lt;/p&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;
+SẢN PHẨM TRONG COMBO&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/goi-co-sang-che-doctorloan-f4/"&gt;– Gối cổ sáng chế DoctorLoan F4: 7.624.000 vnđ&lt;/a&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/goi-lung-sang-che-doctorloan-f3/"&gt;– Gối lưng sáng chế DoctorLoan F3: 3.737.000 vnđ&lt;/a&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/dong-xuan-1ghe-sang-che-doctorloan-n85-chan-dai/"&gt;-Ghế sáng chế DoctorLoan N85 CHÂN NGẮN: 2.127.000 vnđ&lt;/a&gt;&lt;/h1&gt;</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J18" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="K18" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr"/>
+      <c r="M18" s="2" t="inlineStr"/>
+      <c r="N18" s="2" t="inlineStr"/>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>Gói Combo</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr"/>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr"/>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>combo-nan-chinh-co-ban</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>COMBO Nắn Chỉnh Cơ Bản (Toàn Diện)</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="n">
+        <v>19488000</v>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2026/08/1769501593394-77631817-Combonanchinhcoban1.webp</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/combo-nan-chinh-co-ban/</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Nắn chỉnh cơ bản với giải pháp DoctorLoan – Gối sáng chế DoctorLoan: Nắn chỉnh chuyên sâu cột sống cổ và cột sống lưng – Đệm ngồi sáng chế DoctorLoan: nắn chỉnh chuyên sâu xương cùng, xương cụt, xương chậu. – Ghế sáng chế DoctorLoan N85: Giữ dáng ngồi chuẩn trong các sinh hoạt hằng ngày&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;strong&gt;DoctorLoan&lt;/strong&gt; mang đến giải pháp hỗ trợ tư thế và chăm sóc cột sống thông qua hệ thống sản phẩm được thiết kế chuyên biệt cho từng vùng cơ thể.&lt;/p&gt;
+&lt;h3&gt;Gối sáng chế DoctorLoan&lt;/h3&gt;
+&lt;figure id="attachment_4948-2" aria-describedby="caption-attachment-4948-2" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4948 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140497963-707220928-goi-co-doctorloan-f4-3-1000x1000-1-800x800.jpg" alt="Gối cổ sáng chế DoctorLoan F4" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4948-2" class="wp-caption-text"&gt;Gối cổ sáng chế DoctorLoan F4&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;Hỗ trợ &lt;strong&gt;nắn chỉnh chuyên sâu cột sống cổ và cột sống lưng&lt;/strong&gt;, giúp định hướng tư thế phù hợp trong quá trình nghỉ ngơi và sinh hoạt.&lt;/p&gt;
+&lt;h3&gt;Đệm ngồi sáng chế DoctorLoan&lt;/h3&gt;
+&lt;figure id="attachment_4957" aria-describedby="caption-attachment-4957" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4957 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768818488781-178345811-dem-doctorloan-0-1000x1000-1-800x800.jpg" alt="Đệm ngồi sáng chế DoctorLoan" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4957" class="wp-caption-text"&gt;Đệm ngồi sáng chế DoctorLoan&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;Tập trung hỗ trợ &lt;strong&gt;xương cùng, xương cụt và xương chậu&lt;/strong&gt;, giúp duy trì tư thế ngồi phù hợp, đặc biệt với những người thường xuyên phải ngồi lâu.&lt;/p&gt;
+&lt;h3&gt;Ghế sáng chế DoctorLoan N85&lt;/h3&gt;
+&lt;figure id="attachment_4943" aria-describedby="caption-attachment-4943" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4943 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140202131-796146365-ghe-doctorloan-N85-4-1000x1000-1-800x800.jpg" alt="Ghế sáng chế DoctorLoan N85" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4943" class="wp-caption-text"&gt;Ghế sáng chế DoctorLoan N85&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;Hỗ trợ &lt;strong&gt;giữ dáng ngồi chuẩn trong các hoạt động sinh hoạt hằng ngày&lt;/strong&gt;, góp phần hình thành thói quen ngồi khoa học và chủ động chăm sóc cột sống.&lt;/p&gt;
+&lt;p&gt;&lt;strong&gt;DoctorLoan – giải pháp hỗ trợ tư thế, đồng hành cùng bạn chăm sóc cột sống mỗi ngày.&lt;/strong&gt;&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;Link chi tiết về sản phẩm trong Combo Văn Phòng 1&lt;/strong&gt;&lt;/h3&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;–&lt;a href="https://bsthaocotsong.com/san-pham/goi-co-sang-che-doctorloan-f4/"&gt; Gối cổ sáng chế DoctorLoan F4: 7.624.000 vnđ&lt;/a&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/goi-lung-sang-che-doctorloan-f3/"&gt;– Gối lưng sáng chế DoctorLoan F3: 3.737.000 vnđ&lt;/a&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/dem-sang-che-doctorloan/"&gt;– Đệm sáng chế DoctorLoan: 6.000.000 vnđ &lt;/a&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;a href="https://bsthaocotsong.com/san-pham/ghe-sang-che-doctorloan-n85-chan-ngan/"&gt;– Ghế sáng chế DoctorLoan N85 CHÂN NGẮN: 2.127.000 vnđ &lt;/a&gt;&lt;/h1&gt;
+&lt;p&gt; &lt;/p&gt;</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J19" s="2" t="n">
+        <v>18</v>
+      </c>
+      <c r="K19" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr"/>
+      <c r="M19" s="2" t="inlineStr"/>
+      <c r="N19" s="2" t="inlineStr"/>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>Gói Combo</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr"/>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr"/>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>combo-van-phong-1</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>COMBO Văn Phòng 1</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="n">
+        <v>33187000</v>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2026/08/1768833077975-164285146-Combovanphong3.webp</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr"/>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/combo-van-phong-1/</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dành cho những người chuyên ngồi làm việc như dân văn phòng, học sinh, sinh viên, thợ may, phun xăm, nail….&lt;/p&gt;
+&lt;h2&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;GIẢI PHÁP HỖ TRỢ TƯ THẾ NGỒI VÀ CHĂM SÓC CỘT SỐNG DOCTORLOAN&lt;/span&gt;&lt;/strong&gt;&lt;/h2&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Đối với những người phải ngồi làm việc trong thời gian dài như &lt;strong&gt;nhân viên văn phòng, học sinh, sinh viên, thợ may, kỹ thuật viên phun xăm, nhân viên nail&lt;/strong&gt; và nhiều ngành nghề khác, việc duy trì tư thế ngồi phù hợp đóng vai trò quan trọng trong quá trình chăm sóc sức khỏe cột sống.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Thấu hiểu nhu cầu đó, &lt;strong&gt;DoctorLoan&lt;/strong&gt; phát triển các sản phẩm hỗ trợ tư thế ngồi và chăm sóc cột sống, giúp người dùng duy trì tư thế phù hợp trong công việc và sinh hoạt hằng ngày.&lt;/span&gt;&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;1. Ghế sáng chế DoctorLoan 90 – Hỗ trợ tư thế ngồi chuẩn khi làm việc&lt;/span&gt;&lt;/strong&gt;&lt;/h3&gt;
+&lt;p&gt;&lt;img class="aligncenter wp-image-4942 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140315535-147315026-ghe-doctorloan-90D-4-1000x1000-1-800x800.jpg" alt="" width="800" height="800" /&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;&lt;strong&gt;Ghế sáng chế DoctorLoan 90&lt;/strong&gt; được thiết kế dành cho những người thường xuyên phải ngồi làm việc trong thời gian dài.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Sản phẩm tập trung hỗ trợ người sử dụng &lt;strong&gt;duy trì tư thế ngồi thẳng&lt;/strong&gt;, đồng thời tác động hỗ trợ định hướng tư thế tại các vùng &lt;strong&gt;cột sống lưng, xương cùng – xương cụt và xương chậu&lt;/strong&gt;.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;DoctorLoan 90 phù hợp với nhiều đối tượng thường xuyên làm việc ở tư thế ngồi như:&lt;/span&gt;&lt;/p&gt;
+&lt;ul data-spread="false"&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Nhân viên văn phòng, người làm việc với máy tính.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Học sinh, sinh viên phải ngồi học nhiều giờ.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Thợ may, người làm việc tại bàn.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Kỹ thuật viên phun xăm, nhân viên nail.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Những người có đặc thù công việc phải ngồi lâu mỗi ngày.&lt;/span&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Việc sử dụng ghế phù hợp có thể giúp người dùng &lt;strong&gt;ý thức hơn về tư thế ngồi&lt;/strong&gt;, từ đó hình thành thói quen ngồi khoa học và thoải mái hơn trong quá trình làm việc.&lt;/span&gt;&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;2. Gối sáng chế DoctorLoan – Hỗ trợ chăm sóc cột sống cổ và lưng&lt;/span&gt;&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4944" aria-describedby="caption-attachment-4944" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4944 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140445042-521234568-goi-lung-doctorloan-f3-5-1000x1000-1-800x800.jpg" alt="Gỗi lưng sáng chế" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4944" class="wp-caption-text"&gt;Gỗi lưng sáng chế&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;figure id="attachment_4945" aria-describedby="caption-attachment-4945" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4945 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1767577012969-211026264-goi-co-doctorloan-f4-2-1000x1000-1-800x800.jpg" alt="Gỗi cổ sáng chế" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4945" class="wp-caption-text"&gt;Gỗi cổ sáng chế&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Bên cạnh ghế ngồi, &lt;strong&gt;Gối sáng chế DoctorLoan&lt;/strong&gt; được phát triển nhằm hỗ trợ tư thế và chăm sóc chuyên sâu hơn cho vùng &lt;strong&gt;cột sống cổ và cột sống lưng&lt;/strong&gt;.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Thiết kế của sản phẩm hướng đến việc hỗ trợ nâng đỡ và định hướng tư thế phù hợp, giúp người dùng có thêm một giải pháp chăm sóc cột sống trong quá trình nghỉ ngơi và sinh hoạt.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Đây là sản phẩm có thể kết hợp cùng các giải pháp hỗ trợ tư thế khác của DoctorLoan để tạo thành một hệ thống chăm sóc cột sống toàn diện hơn.&lt;/span&gt;&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;3. Ghế sáng chế DoctorLoan N85 – Hỗ trợ duy trì dáng ngồi chuẩn trong sinh hoạt&lt;/span&gt;&lt;/strong&gt;&lt;/h3&gt;
+&lt;p&gt;&lt;img class="aligncenter wp-image-4943 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140202131-796146365-ghe-doctorloan-N85-4-1000x1000-1-800x800.jpg" alt="" width="800" height="800" /&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;&lt;strong&gt;DoctorLoan N85&lt;/strong&gt; là giải pháp được thiết kế nhằm hỗ trợ người dùng &lt;strong&gt;duy trì dáng ngồi phù hợp trong các hoạt động sinh hoạt hằng ngày&lt;/strong&gt;.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Với thiết kế hướng đến sự tiện lợi và khả năng ứng dụng trong nhiều hoàn cảnh, N85 phù hợp với những người mong muốn chủ động xây dựng thói quen giữ tư thế đúng trong cuộc sống.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Sản phẩm đặc biệt hữu ích đối với những người thường xuyên phải ngồi trong thời gian dài hoặc có thói quen ngồi chưa phù hợp.&lt;/span&gt;&lt;/p&gt;
+&lt;h2&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;DoctorLoan – Chủ động chăm sóc cột sống từ tư thế hằng ngày&lt;/span&gt;&lt;/strong&gt;&lt;/h2&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Cột sống đồng hành cùng chúng ta trong mọi hoạt động, từ làm việc, học tập đến nghỉ ngơi và sinh hoạt. Vì vậy, &lt;strong&gt;chăm sóc cột sống không chỉ bắt đầu khi xuất hiện vấn đề mà nên được quan tâm từ những thói quen hằng ngày&lt;/strong&gt;, đặc biệt là tư thế ngồi.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Các sản phẩm sáng chế DoctorLoan như &lt;strong&gt;Ghế DoctorLoan 90, Gối DoctorLoan và Ghế DoctorLoan N85&lt;/strong&gt; hướng đến việc hỗ trợ người dùng duy trì tư thế phù hợp, nâng cao ý thức chăm sóc cột sống và xây dựng thói quen sinh hoạt khoa học hơn.&lt;/span&gt;&lt;/p&gt;
+&lt;p&gt;&lt;span style="color: #000000"&gt;Nếu bạn thường xuyên phải &lt;strong&gt;ngồi làm việc, ngồi học hoặc thực hiện các công việc đòi hỏi tư thế ngồi trong thời gian dài&lt;/strong&gt;, hãy tìm hiểu giải pháp phù hợp từ DoctorLoan để chủ động chăm sóc cột sống mỗi ngày.&lt;/span&gt;&lt;/p&gt;
+&lt;h2&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;Link chi tiết về sản phẩm trong Combo Văn Phòng 1&lt;/span&gt;&lt;/strong&gt;&lt;/h2&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;span style="color: #000000"&gt;&lt;a style="color: #000000" href="https://bsthaocotsong.com/san-pham/goi-co-sang-che-doctorloan-f4/"&gt;– Gối cổ sáng chế DoctorLoan F4: 7.624.000 vnđ&lt;/a&gt;&lt;/span&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;span style="color: #000000"&gt;&lt;a style="color: #000000" href="https://bsthaocotsong.com/san-pham/goi-lung-sang-che-doctorloan-f4/"&gt;– Gối lưng sáng chế DoctorLoan F4: 3.737.000 vnđ&lt;/a&gt;&lt;/span&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;span style="color: #000000"&gt;–&lt;a style="color: #000000" href="https://bsthaocotsong.com/san-pham/ghe-sang-che-doctorloan-n85-chan-ngan/"&gt; Ghế sáng chế DoctorLoan N85 CHÂN NGẮN: 2.127.000 vnđ&lt;/a&gt;&lt;/span&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;span style="color: #000000"&gt;&lt;a style="color: #000000" href="https://bsthaocotsong.com/san-pham/ghe-sang-che-doctorloan-90t-dem-mong/"&gt;– Ghế sáng chế DoctorLoan 90T (đệm mỏng): 19.699.000 vnđ&lt;/a&gt;&lt;/span&gt;&lt;/h1&gt;</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J20" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="K20" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
+      <c r="N20" s="2" t="inlineStr"/>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>Gói Combo</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr"/>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr"/>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>combo-van-phong-2</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>COMBO Văn Phòng 2</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="n">
+        <v>48425000</v>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>VND</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/wp-content/uploads/2026/08/1768833187985-624396734-Combovanphong1.webp</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr"/>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>https://hongcotsong.com/san-pham/combo-van-phong-2/</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>&lt;p&gt;Dành cho những người chuyên ngồi làm việc như dân văn phòng, học sinh, sinh viên, thợ may, phun xăm, nail…. – Ghế sáng chế DoctorLoan 90: giúp giữ thẳng tư thế khi ngồi làm việc đồng thời tập trung nắn chỉnh cột sống lưng, xương cùng xương cụt và xương chậu. – Gối sáng chế DoctorLoan: Nắn chỉnh chuyên sâu cột sống cổ và cột sống lưng – Ghế sáng chế DoctorLoan N85: Giữ dáng ngồi chuẩn trong các sinh hoạt hằng ngày&lt;/p&gt;
+&lt;h2&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;Dành cho người thường xuyên ngồi làm việc, học tập trong thời gian dài&lt;/span&gt;&lt;/strong&gt;&lt;/h2&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Trong cuộc sống hiện đại, nhiều người phải duy trì tư thế ngồi trong nhiều giờ mỗi ngày. Từ &lt;strong&gt;nhân viên văn phòng, học sinh, sinh viên&lt;/strong&gt; đến &lt;strong&gt;thợ may, kỹ thuật viên phun xăm, nhân viên nail&lt;/strong&gt; và những công việc đặc thù khác, việc ngồi lâu và duy trì một tư thế chưa phù hợp có thể khiến cơ thể dễ rơi vào trạng thái mệt mỏi, căng cứng và khó chịu.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Chính vì vậy, việc &lt;strong&gt;chủ động xây dựng tư thế ngồi khoa học và chăm sóc cột sống mỗi ngày&lt;/strong&gt; ngày càng được nhiều người quan tâm.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;DoctorLoan mang đến hệ thống các sản phẩm hỗ trợ tư thế và chăm sóc cột sống, được thiết kế để đồng hành cùng người dùng trong công việc, học tập cũng như các hoạt động sinh hoạt hằng ngày.&lt;/span&gt;&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;Ghế sáng chế DoctorLoan 90 – Hỗ trợ duy trì tư thế ngồi thẳng&lt;/span&gt;&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4951" aria-describedby="caption-attachment-4951" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4951 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140315535-147315026-ghe-doctorloan-90D-4-1000x1000-1-1-800x800.jpg" alt="Ghế sáng chế DoctorLoan 90D (đệm dày)" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4951" class="wp-caption-text"&gt;Ghế sáng chế DoctorLoan 90D (đệm dày)&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;&lt;strong&gt;Ghế sáng chế DoctorLoan 90&lt;/strong&gt; được thiết kế dành cho những người thường xuyên phải ngồi làm việc, học tập trong thời gian dài.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Sản phẩm hỗ trợ người sử dụng &lt;strong&gt;duy trì tư thế ngồi thẳng và ổn định&lt;/strong&gt;, đồng thời tập trung hỗ trợ định hướng tư thế tại các vùng &lt;strong&gt;cột sống lưng, xương cùng – xương cụt và xương chậu&lt;/strong&gt;.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Nhờ thiết kế hướng đến tư thế ngồi khoa học, DoctorLoan 90 có thể trở thành lựa chọn phù hợp cho:&lt;/span&gt;&lt;/p&gt;
+&lt;ul data-spread="false"&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Nhân viên văn phòng thường xuyên làm việc với máy tính.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Học sinh, sinh viên ngồi học nhiều giờ mỗi ngày.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Thợ may và những người làm việc tại bàn.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Kỹ thuật viên phun xăm.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Nhân viên nail.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;Người có đặc thù công việc phải ngồi lâu.&lt;/span&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;DoctorLoan 90 – hỗ trợ tư thế ngồi đúng, đồng hành cùng bạn trong từng giờ làm việc và học tập.&lt;/span&gt;&lt;/strong&gt;&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;Gối sáng chế DoctorLoan – Hỗ trợ tư thế vùng cổ và cột sống lưng&lt;/span&gt;&lt;/strong&gt;&lt;/h3&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Bên cạnh giải pháp dành cho tư thế ngồi, &lt;strong&gt;Gối sáng chế DoctorLoan&lt;/strong&gt; được phát triển nhằm hỗ trợ chăm sóc &lt;strong&gt;cột sống cổ và cột sống lưng&lt;/strong&gt;.&lt;/span&gt;&lt;/p&gt;
+&lt;figure id="attachment_4948" aria-describedby="caption-attachment-4948" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4948 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140497963-707220928-goi-co-doctorloan-f4-3-1000x1000-1-800x800.jpg" alt="Gối cổ sáng chế DoctorLoan F4" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4948" class="wp-caption-text"&gt;Gối cổ sáng chế DoctorLoan F4&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Thiết kế của sản phẩm hướng đến việc hỗ trợ cơ thể duy trì tư thế phù hợp, tập trung vào các vùng cột sống quan trọng trong quá trình nghỉ ngơi và sinh hoạt.&lt;/span&gt;&lt;/p&gt;
+&lt;figure id="attachment_4949" aria-describedby="caption-attachment-4949" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4949 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140443068-271317917-goi-lung-doctorloan-f3-4-1000x1000-1-800x800.jpg" alt="Gối lưng sáng chế DoctorLoan F3" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4949" class="wp-caption-text"&gt;Gối lưng sáng chế DoctorLoan F3&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Với những người thường xuyên làm việc ở tư thế ngồi, sử dụng máy tính hoặc có cường độ học tập cao, việc kết hợp các giải pháp hỗ trợ tư thế trong sinh hoạt hằng ngày có thể giúp hình thành thói quen chăm sóc cột sống một cách chủ động hơn.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Gối DoctorLoan – giải pháp hỗ trợ chăm sóc cột sống cổ và lưng trong cuộc sống hằng ngày.&lt;/span&gt;&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;Ghế sáng chế DoctorLoan N85 – Hỗ trợ duy trì dáng ngồi chuẩn trong sinh hoạt&lt;/span&gt;&lt;/strong&gt;&lt;/h3&gt;
+&lt;figure id="attachment_4950" aria-describedby="caption-attachment-4950" style="width: 800px" class="wp-caption aligncenter"&gt;&lt;img class="wp-image-4950 size-large" src="https://bsthaocotsong.com/wp-content/uploads/2026/08/1768140199100-761249413-ghe-doctorloan-N85-3-1000x1000-1-800x800.jpg" alt="Ghế sáng chế DoctorLoan N85 CHÂN NGẮN" width="800" height="800" /&gt;&lt;figcaption id="caption-attachment-4950" class="wp-caption-text"&gt;Ghế sáng chế DoctorLoan N85 CHÂN NGẮN&lt;/figcaption&gt;&lt;/figure&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;&lt;strong&gt;Ghế sáng chế DoctorLoan N85&lt;/strong&gt; được thiết kế để hỗ trợ người dùng &lt;strong&gt;duy trì dáng ngồi phù hợp trong các hoạt động sinh hoạt hằng ngày&lt;/strong&gt;.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Không chỉ dành cho thời gian làm việc, N85 hướng đến việc giúp người dùng chú ý hơn đến tư thế trong nhiều hoạt động khác nhau, từ ngồi nghỉ ngơi, trò chuyện đến các sinh hoạt thường nhật.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Đây là lựa chọn phù hợp cho những người mong muốn xây dựng &lt;strong&gt;thói quen ngồi khoa học&lt;/strong&gt;, chủ động quan tâm đến tư thế và chăm sóc cột sống lâu dài.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;DoctorLoan N85 – hỗ trợ duy trì dáng ngồi phù hợp trong từng hoạt động hằng ngày.&lt;/span&gt;&lt;/p&gt;
+&lt;h2&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;DoctorLoan – Chủ động chăm sóc cột sống bắt đầu từ tư thế&lt;/span&gt;&lt;/strong&gt;&lt;/h2&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Cột sống đóng vai trò quan trọng trong khả năng vận động và các hoạt động thường ngày. Tuy nhiên, chúng ta thường chỉ quan tâm đến cột sống khi cơ thể xuất hiện cảm giác khó chịu.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Thay vì chờ đến khi vấn đề xuất hiện, mỗi người có thể bắt đầu từ những điều đơn giản như &lt;strong&gt;chú ý tư thế khi ngồi, thay đổi tư thế sau thời gian dài và xây dựng thói quen sinh hoạt khoa học&lt;/strong&gt;.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Với hệ thống sản phẩm gồm &lt;strong&gt;Ghế DoctorLoan 90, Gối DoctorLoan và Ghế DoctorLoan N85&lt;/strong&gt;, DoctorLoan hướng đến việc cung cấp các giải pháp hỗ trợ tư thế phù hợp với nhiều nhu cầu khác nhau trong cuộc sống.&lt;/span&gt;&lt;/p&gt;
+&lt;p class="isSelectedEnd"&gt;&lt;span style="color: #000000"&gt;Dù bạn là &lt;strong&gt;dân văn phòng, học sinh, sinh viên, thợ may, kỹ thuật viên phun xăm, nhân viên nail&lt;/strong&gt; hay thường xuyên phải ngồi trong thời gian dài, việc lựa chọn một giải pháp hỗ trợ tư thế phù hợp có thể là bước khởi đầu để bạn quan tâm hơn đến sức khỏe cột sống mỗi ngày.&lt;/span&gt;&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;&lt;span style="color: #000000"&gt;Lựa chọn giải pháp DoctorLoan phù hợp với nhu cầu của bạn&lt;/span&gt;&lt;/strong&gt;&lt;/h3&gt;
+&lt;ul data-spread="false"&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;&lt;strong&gt;DoctorLoan 90:&lt;/strong&gt; Hỗ trợ duy trì tư thế ngồi thẳng, tập trung vào vùng cột sống lưng, xương cùng – xương cụt và xương chậu.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;&lt;strong&gt;Gối DoctorLoan:&lt;/strong&gt; Hỗ trợ chăm sóc và định hướng tư thế vùng cột sống cổ và cột sống lưng.&lt;/span&gt;&lt;/li&gt;
+&lt;li&gt;&lt;span style="color: #000000"&gt;&lt;strong&gt;DoctorLoan N85:&lt;/strong&gt; Hỗ trợ duy trì dáng ngồi phù hợp trong các hoạt động sinh hoạt hằng ngày.&lt;/span&gt;&lt;/li&gt;
+&lt;/ul&gt;
+&lt;p&gt;&lt;span style="color: #000000"&gt;DoctorLoan – đồng hành cùng bạn xây dựng tư thế khoa học và chủ động chăm sóc cột sống mỗi ngày.&lt;/span&gt;&lt;/p&gt;
+&lt;h3&gt;&lt;strong&gt;Link chi tiết về sản phẩm trong Combo Văn Phòng 1:&lt;/strong&gt;&lt;/h3&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;span style="color: #000000"&gt;&lt;a style="color: #000000" href="https://bsthaocotsong.com/san-pham/goi-co-sang-che-doctorloan-f4/"&gt;– Gối cổ sáng chế DoctorLoan F4: 7.624.000 vnđ&lt;/a&gt;&lt;/span&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;span style="color: #000000"&gt;&lt;a style="color: #000000" href="https://bsthaocotsong.com/san-pham/goi-lung-sang-che-doctorloan-f3/"&gt;– Gối lưng sáng chế DoctorLoan F3: 3.737.000 vnđ&lt;/a&gt;&lt;/span&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;span style="color: #000000"&gt;&lt;a style="color: #000000" href="https://bsthaocotsong.com/san-pham/ghe-sang-che-doctorloan-n85-chan-ngan/"&gt;– Ghế sáng chế DoctorLoan N85 CHÂN NGẮN: 2.127.000 vnđ&lt;/a&gt;&lt;/span&gt;&lt;/h1&gt;
+&lt;h1 class="text-2xl md:text-3xl font-bold text-gray-900 leading-tight break-words"&gt;&lt;span style="color: #000000"&gt;&lt;a style="color: #000000" href="https://bsthaocotsong.com/san-pham/4469/"&gt;– Ghế sáng chế DoctorLoan 90D (đệm dày): 34.937.000 vnđ&lt;/a&gt;&lt;/span&gt;&lt;/h1&gt;</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="J21" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="K21" s="2" t="inlineStr">
+        <is>
+          <t>Đặt mua ngay</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr"/>
+      <c r="M21" s="2" t="inlineStr"/>
+      <c r="N21" s="2" t="inlineStr"/>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>card</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>Gói Combo</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr"/>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>Chat tư vấn</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr"/>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>open-chat-trigger</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>